<commit_message>
Add MA02 Management Attestation to scope evidence and space evidence references
- Restore the Management Attestation email (Frank Puentes, 08/18/2026) as
  MA02 in 01_Management_Attestation_In-Scope_Applications and cite it under
  Applications in Scope Identified for all 10 samples (attached signed
  attestation section 2 lists the 13 in-scope applications).
- Separate every evidence reference with a blank line on the testing tab,
  Evidence Map and WP Summary; space the observations in column Q.
- Widen testing columns so the application rows fit on screen.
- Evidence Index, removal log, README, zip and Word guide updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01884Wo9yAWN5dtHStWCWnty
</commit_message>
<xml_diff>
--- a/BSI.IT.6.C7.3-Evidences/BSI.IT.6.C7.3_E00_Workpaper_DR_DIV_INTEGRATED_APPLICATION_Evidence.xlsx
+++ b/BSI.IT.6.C7.3-Evidences/BSI.IT.6.C7.3_E00_Workpaper_DR_DIV_INTEGRATED_APPLICATION_Evidence.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BSI.IT.6.C7.3 Evidence Index" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'BSI.IT.6.C7.3 Evidence Index'!$A$2:$K$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'BSI.IT.6.C7.3 Evidence Index'!$A$2:$K$34</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -1422,7 +1422,9 @@
       </c>
       <c r="B9" s="51" t="inlineStr">
         <is>
-          <t>MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png; E01 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx</t>
+          <t>MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png
+MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg
+E01 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx</t>
         </is>
       </c>
       <c r="C9" s="51" t="n"/>
@@ -1440,7 +1442,8 @@
       </c>
       <c r="B10" s="51" t="inlineStr">
         <is>
-          <t>E03 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls; E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+          <t>E03 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls
+E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
         </is>
       </c>
       <c r="C10" s="51" t="n"/>
@@ -1535,7 +1538,10 @@
       </c>
       <c r="F14" s="51" t="inlineStr">
         <is>
-          <t>MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png; E01 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx; E02</t>
+          <t>MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png
+MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg
+E01 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx
+E02 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg</t>
         </is>
       </c>
       <c r="G14" s="53" t="inlineStr">
@@ -1575,7 +1581,9 @@
       </c>
       <c r="F15" s="51" t="inlineStr">
         <is>
-          <t>E03 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls; E16b; BLA01–BLA05 (BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email)</t>
+          <t>E03 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls
+E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx
+BLA01–BLA05 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email</t>
         </is>
       </c>
       <c r="G15" s="53" t="inlineStr">
@@ -1615,7 +1623,10 @@
       </c>
       <c r="F16" s="51" t="inlineStr">
         <is>
-          <t>BLA01–BLA06 (BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email); DMA01–DMA12 (BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals); E09; E03 approval fields</t>
+          <t>BLA01–BLA06 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email
+DMA01–DMA12 – BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals
+E09 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg
+E03 – approval fields</t>
         </is>
       </c>
       <c r="G16" s="53" t="inlineStr">
@@ -1655,7 +1666,10 @@
       </c>
       <c r="F17" s="51" t="inlineStr">
         <is>
-          <t>E04, E02, MA01 (BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence / 01_Management_Attestation_In-Scope_Applications); E03 / E16b source data</t>
+          <t>E04 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg
+E02 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg
+MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png
+E03 / E16b – source data</t>
         </is>
       </c>
       <c r="G17" s="55" t="inlineStr">
@@ -2209,24 +2223,24 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="10" customWidth="1" style="71" min="1" max="1"/>
-    <col width="60" customWidth="1" style="71" min="2" max="2"/>
-    <col width="55" customWidth="1" style="71" min="3" max="3"/>
-    <col width="60" customWidth="1" style="71" min="4" max="4"/>
-    <col width="60" customWidth="1" style="71" min="5" max="5"/>
-    <col width="62" customWidth="1" style="71" min="6" max="7"/>
-    <col width="55" customWidth="1" style="71" min="7" max="7"/>
-    <col width="58" customWidth="1" style="71" min="8" max="8"/>
-    <col width="62" customWidth="1" style="71" min="9" max="9"/>
-    <col width="62" customWidth="1" style="71" min="10" max="10"/>
-    <col width="60" customWidth="1" style="71" min="11" max="11"/>
-    <col width="60" customWidth="1" style="71" min="12" max="12"/>
-    <col width="66" customWidth="1" style="71" min="13" max="13"/>
-    <col width="66" customWidth="1" style="71" min="14" max="14"/>
-    <col width="66" customWidth="1" style="71" min="15" max="15"/>
-    <col hidden="1" width="58" customWidth="1" style="71" min="16" max="16"/>
-    <col width="70" customWidth="1" style="71" min="17" max="17"/>
-    <col width="95" customWidth="1" style="71" min="18" max="18"/>
-    <col width="48" customWidth="1" style="57" min="19" max="19"/>
+    <col width="90" customWidth="1" style="71" min="2" max="2"/>
+    <col width="90" customWidth="1" style="71" min="3" max="3"/>
+    <col width="90" customWidth="1" style="71" min="4" max="4"/>
+    <col width="90" customWidth="1" style="71" min="5" max="5"/>
+    <col width="90" customWidth="1" style="71" min="6" max="7"/>
+    <col width="90" customWidth="1" style="71" min="7" max="7"/>
+    <col width="90" customWidth="1" style="71" min="8" max="8"/>
+    <col width="90" customWidth="1" style="71" min="9" max="9"/>
+    <col width="90" customWidth="1" style="71" min="10" max="10"/>
+    <col width="90" customWidth="1" style="71" min="11" max="11"/>
+    <col width="90" customWidth="1" style="71" min="12" max="12"/>
+    <col width="90" customWidth="1" style="71" min="13" max="13"/>
+    <col width="90" customWidth="1" style="71" min="14" max="14"/>
+    <col width="90" customWidth="1" style="71" min="15" max="15"/>
+    <col hidden="1" width="90" customWidth="1" style="71" min="16" max="16"/>
+    <col width="90" customWidth="1" style="71" min="17" max="17"/>
+    <col width="160" customWidth="1" style="71" min="18" max="18"/>
+    <col width="50" customWidth="1" style="57" min="19" max="19"/>
     <col width="8.6640625" customWidth="1" style="57" min="20" max="65"/>
   </cols>
   <sheetData>
@@ -2393,7 +2407,7 @@
       <c r="BM4" s="58" t="n"/>
       <c r="BN4" s="58" t="n"/>
     </row>
-    <row r="5" ht="332" customFormat="1" customHeight="1" s="47">
+    <row r="5" ht="404" customFormat="1" customHeight="1" s="47">
       <c r="A5" s="45" t="n">
         <v>1822</v>
       </c>
@@ -2521,9 +2535,10 @@
       </c>
       <c r="N5" s="69" t="inlineStr">
         <is>
-          <t>PASS – ACH Express is identified as in scope. The BCiC in-scope applications view (BSI In-Scope Applications-2026) shows App ID 1822 selected among the 10 applications flagged 2025 Backup/Restore DIV Scope = True; corroborated by the BCiC DR-scope export, the IT BIA/applications review and the management attestation.
+          <t>PASS – ACH Express is identified as in scope. The BCiC in-scope applications view BSI In-Scope Applications-2026 (MA01, Management_Attestation folder) shows App ID 1822 selected among the 10 applications flagged 2025 Backup/Restore DIV Scope = True, and the signed Management Attestation (MA02, §2) lists it among the 13 in-scope applications that store business data; corroborated by the BCiC DR-scope export (E01, E02), the IT BIA/applications review (E05) and the signed attestations (MA02, DMA02).
 Evidence location (BSI.IT.6.C7.3-Evidences):
 • MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png – BSI In-Scope Applications-2026 – App ID 1822 selected; 2025 DR Test Scope, 2025 Backup/Restore Test Scope and 2025 Backup/Restore DIV Scope = True
+• MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg – Management Attestation email 08/18/2026 – attached signed attestation (4069_001.pdf) §2 lists the 13 in-scope applications that store business data, including this application
 • E01 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx – row 3 – 2025 DR Test Scope = True; 2025 Backup/Restore DIV Scope = True
 • E02 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg – view 'Applications In Scope for DR Test BSI'
 • E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg – BIA results &amp; applications list review
@@ -2561,8 +2576,9 @@
       </c>
       <c r="R5" s="68" t="inlineStr">
         <is>
-          <t>[01 Management Attestation / In-Scope Applications]
+          <t xml:space="preserve">[01 Management Attestation / In-Scope Applications]
 MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png
+MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg
 [02 Business Line Approval Results – Email]
 BLA01 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf
 [03 DIV Manager Attestation Email Approvals]
@@ -2575,7 +2591,8 @@
 E04 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg
 E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg
 E09 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg
-E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx
+</t>
         </is>
       </c>
       <c r="S5" s="42" t="inlineStr">
@@ -2631,7 +2648,7 @@
       <c r="BM5" s="58" t="n"/>
       <c r="BN5" s="58" t="n"/>
     </row>
-    <row r="6" ht="332" customFormat="1" customHeight="1" s="39">
+    <row r="6" ht="404" customFormat="1" customHeight="1" s="39">
       <c r="A6" s="45" t="n">
         <v>1867</v>
       </c>
@@ -2763,9 +2780,10 @@
       </c>
       <c r="N6" s="69" t="inlineStr">
         <is>
-          <t>PASS – FedExport - BSI is identified as in scope. The BCiC in-scope applications view (BSI In-Scope Applications-2026) shows App ID 1867 selected among the 10 applications flagged 2025 Backup/Restore DIV Scope = True; corroborated by the BCiC DR-scope export, the IT BIA/applications review and the management attestation.
+          <t>PASS – FedExport - BSI is identified as in scope. The BCiC in-scope applications view BSI In-Scope Applications-2026 (MA01, Management_Attestation folder) shows App ID 1867 selected among the 10 applications flagged 2025 Backup/Restore DIV Scope = True, and the signed Management Attestation (MA02, §2) lists it among the 13 in-scope applications that store business data; corroborated by the BCiC DR-scope export (E01, E02), the IT BIA/applications review (E05) and the signed attestations (MA02, DMA02).
 Evidence location (BSI.IT.6.C7.3-Evidences):
 • MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png – BSI In-Scope Applications-2026 – App ID 1867 selected; 2025 DR Test Scope, 2025 Backup/Restore Test Scope and 2025 Backup/Restore DIV Scope = True
+• MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg – Management Attestation email 08/18/2026 – attached signed attestation (4069_001.pdf) §2 lists the 13 in-scope applications that store business data, including this application
 • E01 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx – row 19 – 2025 DR Test Scope = True; 2025 Backup/Restore DIV Scope = True
 • E02 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg – view 'Applications In Scope for DR Test BSI'
 • E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg – BIA results &amp; applications list review
@@ -2803,8 +2821,9 @@
       </c>
       <c r="R6" s="43" t="inlineStr">
         <is>
-          <t>[01 Management Attestation / In-Scope Applications]
+          <t xml:space="preserve">[01 Management Attestation / In-Scope Applications]
 MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png
+MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg
 [02 Business Line Approval Results – Email]
 BLA01 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf
 [03 DIV Manager Attestation Email Approvals]
@@ -2817,7 +2836,8 @@
 E04 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg
 E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg
 E09 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg
-E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx
+</t>
         </is>
       </c>
       <c r="S6" s="42" t="inlineStr">
@@ -2873,7 +2893,7 @@
       <c r="BM6" s="58" t="n"/>
       <c r="BN6" s="58" t="n"/>
     </row>
-    <row r="7" ht="332" customFormat="1" customHeight="1" s="39">
+    <row r="7" ht="404" customFormat="1" customHeight="1" s="39">
       <c r="A7" s="45" t="n">
         <v>1868</v>
       </c>
@@ -3005,9 +3025,10 @@
       </c>
       <c r="N7" s="69" t="inlineStr">
         <is>
-          <t>PASS – FedImport - BSI is identified as in scope. The BCiC in-scope applications view (BSI In-Scope Applications-2026) shows App ID 1868 selected among the 10 applications flagged 2025 Backup/Restore DIV Scope = True; corroborated by the BCiC DR-scope export, the IT BIA/applications review and the management attestation.
+          <t>PASS – FedImport - BSI is identified as in scope. The BCiC in-scope applications view BSI In-Scope Applications-2026 (MA01, Management_Attestation folder) shows App ID 1868 selected among the 10 applications flagged 2025 Backup/Restore DIV Scope = True, and the signed Management Attestation (MA02, §2) lists it among the 13 in-scope applications that store business data; corroborated by the BCiC DR-scope export (E01, E02), the IT BIA/applications review (E05) and the signed attestations (MA02, DMA02).
 Evidence location (BSI.IT.6.C7.3-Evidences):
 • MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png – BSI In-Scope Applications-2026 – App ID 1868 selected; 2025 DR Test Scope, 2025 Backup/Restore Test Scope and 2025 Backup/Restore DIV Scope = True
+• MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg – Management Attestation email 08/18/2026 – attached signed attestation (4069_001.pdf) §2 lists the 13 in-scope applications that store business data, including this application
 • E01 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx – row 20 – 2025 DR Test Scope = True; 2025 Backup/Restore DIV Scope = True
 • E02 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg – view 'Applications In Scope for DR Test BSI'
 • E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg – BIA results &amp; applications list review
@@ -3044,8 +3065,9 @@
       </c>
       <c r="R7" s="40" t="inlineStr">
         <is>
-          <t>[01 Management Attestation / In-Scope Applications]
+          <t xml:space="preserve">[01 Management Attestation / In-Scope Applications]
 MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png
+MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg
 [02 Business Line Approval Results – Email]
 BLA01 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf
 [03 DIV Manager Attestation Email Approvals]
@@ -3058,7 +3080,8 @@
 E04 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg
 E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg
 E09 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg
-E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx
+</t>
         </is>
       </c>
       <c r="S7" s="42" t="inlineStr">
@@ -3280,9 +3303,10 @@
       </c>
       <c r="N8" s="69" t="inlineStr">
         <is>
-          <t>PASS – Imaging101 is identified as in scope. The BCiC in-scope applications view (BSI In-Scope Applications-2026) shows App ID 3299 selected among the 10 applications flagged 2025 Backup/Restore DIV Scope = True; corroborated by the BCiC DR-scope export, the IT BIA/applications review and the management attestation.
+          <t>PASS – Imaging101 is identified as in scope. The BCiC in-scope applications view BSI In-Scope Applications-2026 (MA01, Management_Attestation folder) shows App ID 3299 selected among the 10 applications flagged 2025 Backup/Restore DIV Scope = True, and the signed Management Attestation (MA02, §2) lists it among the 13 in-scope applications that store business data; corroborated by the BCiC DR-scope export (E01, E02), the IT BIA/applications review (E05) and the signed attestations (MA02, DMA02).
 Evidence location (BSI.IT.6.C7.3-Evidences):
 • MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png – BSI In-Scope Applications-2026 – App ID 3299 selected; 2025 DR Test Scope, 2025 Backup/Restore Test Scope and 2025 Backup/Restore DIV Scope = True
+• MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg – Management Attestation email 08/18/2026 – attached signed attestation (4069_001.pdf) §2 lists the 13 in-scope applications that store business data, including this application
 • E01 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx – row 24 – 2025 DR Test Scope = True; 2025 Backup/Restore DIV Scope = True
 • E02 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg – view 'Applications In Scope for DR Test BSI'
 • E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg – BIA results &amp; applications list review
@@ -3326,8 +3350,9 @@
       </c>
       <c r="R8" s="43" t="inlineStr">
         <is>
-          <t>[01 Management Attestation / In-Scope Applications]
+          <t xml:space="preserve">[01 Management Attestation / In-Scope Applications]
 MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png
+MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg
 [02 Business Line Approval Results – Email]
 BLA01 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf
 BLA02 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf
@@ -3343,7 +3368,8 @@
 E04 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg
 E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg
 E09 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg
-E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx
+</t>
         </is>
       </c>
       <c r="S8" s="42" t="inlineStr">
@@ -3399,7 +3425,7 @@
       <c r="BM8" s="58" t="n"/>
       <c r="BN8" s="58" t="n"/>
     </row>
-    <row r="9" ht="296" customFormat="1" customHeight="1" s="39">
+    <row r="9" ht="356" customFormat="1" customHeight="1" s="39">
       <c r="A9" s="45" t="n">
         <v>4052</v>
       </c>
@@ -3522,9 +3548,10 @@
       </c>
       <c r="N9" s="69" t="inlineStr">
         <is>
-          <t>PASS – Interface Monitor is identified as in scope. The BCiC in-scope applications view (BSI In-Scope Applications-2026) shows App ID 4052 selected among the 10 applications flagged 2025 Backup/Restore DIV Scope = True; corroborated by the BCiC DR-scope export, the IT BIA/applications review and the management attestation.
+          <t>PASS – Interface Monitor is identified as in scope. The BCiC in-scope applications view BSI In-Scope Applications-2026 (MA01, Management_Attestation folder) shows App ID 4052 selected among the 10 applications flagged 2025 Backup/Restore DIV Scope = True, and the signed Management Attestation (MA02, §2) lists it among the 13 in-scope applications that store business data; corroborated by the BCiC DR-scope export (E01, E02), the IT BIA/applications review (E05) and the signed attestations (MA02, DMA02).
 Evidence location (BSI.IT.6.C7.3-Evidences):
 • MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png – BSI In-Scope Applications-2026 – App ID 4052 selected; 2025 DR Test Scope, 2025 Backup/Restore Test Scope and 2025 Backup/Restore DIV Scope = True
+• MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg – Management Attestation email 08/18/2026 – attached signed attestation (4069_001.pdf) §2 lists the 13 in-scope applications that store business data, including this application
 • E01 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx – row 25 – 2025 DR Test Scope = True; 2025 Backup/Restore DIV Scope = True
 • E02 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg – view 'Applications In Scope for DR Test BSI'
 • E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg – BIA results &amp; applications list review
@@ -3561,8 +3588,9 @@
       </c>
       <c r="R9" s="40" t="inlineStr">
         <is>
-          <t>[01 Management Attestation / In-Scope Applications]
+          <t xml:space="preserve">[01 Management Attestation / In-Scope Applications]
 MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png
+MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg
 [02 Business Line Approval Results – Email]
 BLA04 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx
 [03 DIV Manager Attestation Email Approvals]
@@ -3574,7 +3602,8 @@
 E03 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls
 E04 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg
 E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg
-E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx
+</t>
         </is>
       </c>
       <c r="S9" s="42" t="inlineStr">
@@ -3630,7 +3659,7 @@
       <c r="BM9" s="58" t="n"/>
       <c r="BN9" s="58" t="n"/>
     </row>
-    <row r="10" ht="332" customFormat="1" customHeight="1" s="39">
+    <row r="10" ht="380" customFormat="1" customHeight="1" s="39">
       <c r="A10" s="45" t="n">
         <v>3301</v>
       </c>
@@ -3757,9 +3786,10 @@
       </c>
       <c r="N10" s="69" t="inlineStr">
         <is>
-          <t>PASS – MQ Payment Monitor is identified as in scope. The BCiC in-scope applications view (BSI In-Scope Applications-2026) shows App ID 3301 selected among the 10 applications flagged 2025 Backup/Restore DIV Scope = True; corroborated by the BCiC DR-scope export, the IT BIA/applications review and the management attestation.
+          <t>PASS – MQ Payment Monitor is identified as in scope. The BCiC in-scope applications view BSI In-Scope Applications-2026 (MA01, Management_Attestation folder) shows App ID 3301 selected among the 10 applications flagged 2025 Backup/Restore DIV Scope = True, and the signed Management Attestation (MA02, §2) lists it among the 13 in-scope applications that store business data; corroborated by the BCiC DR-scope export (E01, E02), the IT BIA/applications review (E05) and the signed attestations (MA02, DMA02).
 Evidence location (BSI.IT.6.C7.3-Evidences):
 • MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png – BSI In-Scope Applications-2026 – App ID 3301 selected; 2025 DR Test Scope, 2025 Backup/Restore Test Scope and 2025 Backup/Restore DIV Scope = True
+• MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg – Management Attestation email 08/18/2026 – attached signed attestation (4069_001.pdf) §2 lists the 13 in-scope applications that store business data, including this application
 • E01 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx – row 31 – 2025 DR Test Scope = True; 2025 Backup/Restore DIV Scope = True
 • E02 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg – view 'Applications In Scope for DR Test BSI'
 • E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg – BIA results &amp; applications list review
@@ -3795,8 +3825,9 @@
       </c>
       <c r="R10" s="43" t="inlineStr">
         <is>
-          <t>[01 Management Attestation / In-Scope Applications]
+          <t xml:space="preserve">[01 Management Attestation / In-Scope Applications]
 MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png
+MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg
 [02 Business Line Approval Results – Email]
 BLA03 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf
 [03 DIV Manager Attestation Email Approvals]
@@ -3810,7 +3841,8 @@
 E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg
 E07 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg
 E08 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg
-E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx
+</t>
         </is>
       </c>
       <c r="S10" s="42" t="inlineStr">
@@ -3866,7 +3898,7 @@
       <c r="BM10" s="58" t="n"/>
       <c r="BN10" s="58" t="n"/>
     </row>
-    <row r="11" ht="380" customFormat="1" customHeight="1" s="39">
+    <row r="11" ht="409" customFormat="1" customHeight="1" s="39">
       <c r="A11" s="45" t="n">
         <v>1903</v>
       </c>
@@ -4020,9 +4052,10 @@
       </c>
       <c r="N11" s="69" t="inlineStr">
         <is>
-          <t>PASS – OFAC - BSI is identified as in scope. The BCiC in-scope applications view (BSI In-Scope Applications-2026) shows App ID 1903 selected among the 10 applications flagged 2025 Backup/Restore DIV Scope = True; corroborated by the BCiC DR-scope export, the IT BIA/applications review and the management attestation.
+          <t>PASS – OFAC - BSI is identified as in scope. The BCiC in-scope applications view BSI In-Scope Applications-2026 (MA01, Management_Attestation folder) shows App ID 1903 selected among the 10 applications flagged 2025 Backup/Restore DIV Scope = True, and the signed Management Attestation (MA02, §2) lists it among the 13 in-scope applications that store business data; corroborated by the BCiC DR-scope export (E01, E02), the IT BIA/applications review (E05) and the signed attestations (MA02, DMA02).
 Evidence location (BSI.IT.6.C7.3-Evidences):
 • MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png – BSI In-Scope Applications-2026 – App ID 1903 selected; 2025 DR Test Scope, 2025 Backup/Restore Test Scope and 2025 Backup/Restore DIV Scope = True
+• MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg – Management Attestation email 08/18/2026 – attached signed attestation (4069_001.pdf) §2 lists the 13 in-scope applications that store business data, including this application
 • E01 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx – row 34 – 2025 DR Test Scope = True; 2025 Backup/Restore DIV Scope = True
 • E02 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg – view 'Applications In Scope for DR Test BSI'
 • E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg – BIA results &amp; applications list review
@@ -4063,8 +4096,9 @@
       </c>
       <c r="R11" s="40" t="inlineStr">
         <is>
-          <t>[01 Management Attestation / In-Scope Applications]
+          <t xml:space="preserve">[01 Management Attestation / In-Scope Applications]
 MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png
+MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg
 [02 Business Line Approval Results – Email]
 BLA02 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf
 BLA03 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf
@@ -4080,7 +4114,8 @@
 E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg
 E07 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg
 E08 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg
-E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx
+</t>
         </is>
       </c>
       <c r="S11" s="42" t="inlineStr">
@@ -4136,7 +4171,7 @@
       <c r="BM11" s="58" t="n"/>
       <c r="BN11" s="58" t="n"/>
     </row>
-    <row r="12" ht="308" customFormat="1" customHeight="1" s="39">
+    <row r="12" ht="356" customFormat="1" customHeight="1" s="39">
       <c r="A12" s="45" t="n">
         <v>1917</v>
       </c>
@@ -4260,9 +4295,10 @@
       </c>
       <c r="N12" s="69" t="inlineStr">
         <is>
-          <t>PASS – ReconXpert is identified as in scope. The BCiC in-scope applications view (BSI In-Scope Applications-2026) shows App ID 1917 selected among the 10 applications flagged 2025 Backup/Restore DIV Scope = True; corroborated by the BCiC DR-scope export, the IT BIA/applications review and the management attestation.
+          <t>PASS – ReconXpert is identified as in scope. The BCiC in-scope applications view BSI In-Scope Applications-2026 (MA01, Management_Attestation folder) shows App ID 1917 selected among the 10 applications flagged 2025 Backup/Restore DIV Scope = True, and the signed Management Attestation (MA02, §2) lists it among the 13 in-scope applications that store business data; corroborated by the BCiC DR-scope export (E01, E02), the IT BIA/applications review (E05) and the signed attestations (MA02, DMA02).
 Evidence location (BSI.IT.6.C7.3-Evidences):
 • MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png – BSI In-Scope Applications-2026 – App ID 1917 selected; 2025 DR Test Scope, 2025 Backup/Restore Test Scope and 2025 Backup/Restore DIV Scope = True
+• MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg – Management Attestation email 08/18/2026 – attached signed attestation (4069_001.pdf) §2 lists the 13 in-scope applications that store business data, including this application
 • E01 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx – row 36 – 2025 DR Test Scope = True; 2025 Backup/Restore DIV Scope = True
 • E02 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg – view 'Applications In Scope for DR Test BSI'
 • E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg – BIA results &amp; applications list review
@@ -4298,8 +4334,9 @@
       </c>
       <c r="R12" s="43" t="inlineStr">
         <is>
-          <t>[01 Management Attestation / In-Scope Applications]
+          <t xml:space="preserve">[01 Management Attestation / In-Scope Applications]
 MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png
+MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg
 [02 Business Line Approval Results – Email]
 BLA05 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf
 BLA06 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg
@@ -4312,7 +4349,8 @@
 E04 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg
 E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg
 E10 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg
-E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx
+</t>
         </is>
       </c>
       <c r="S12" s="42" t="inlineStr">
@@ -4368,7 +4406,7 @@
       <c r="BM12" s="58" t="n"/>
       <c r="BN12" s="58" t="n"/>
     </row>
-    <row r="13" ht="356" customFormat="1" customHeight="1" s="39">
+    <row r="13" ht="404" customFormat="1" customHeight="1" s="39">
       <c r="A13" s="45" t="n">
         <v>1936</v>
       </c>
@@ -4512,9 +4550,10 @@
       </c>
       <c r="N13" s="69" t="inlineStr">
         <is>
-          <t>PASS – Swift Interface - BSI is identified as in scope. The BCiC in-scope applications view (BSI In-Scope Applications-2026) shows App ID 1936 selected among the 10 applications flagged 2025 Backup/Restore DIV Scope = True; corroborated by the BCiC DR-scope export, the IT BIA/applications review and the management attestation.
+          <t>PASS – Swift Interface - BSI is identified as in scope. The BCiC in-scope applications view BSI In-Scope Applications-2026 (MA01, Management_Attestation folder) shows App ID 1936 selected among the 10 applications flagged 2025 Backup/Restore DIV Scope = True, and the signed Management Attestation (MA02, §2) lists it among the 13 in-scope applications that store business data; corroborated by the BCiC DR-scope export (E01, E02), the IT BIA/applications review (E05) and the signed attestations (MA02, DMA02).
 Evidence location (BSI.IT.6.C7.3-Evidences):
 • MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png – BSI In-Scope Applications-2026 – App ID 1936 selected; 2025 DR Test Scope, 2025 Backup/Restore Test Scope and 2025 Backup/Restore DIV Scope = True
+• MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg – Management Attestation email 08/18/2026 – attached signed attestation (4069_001.pdf) §2 lists the 13 in-scope applications that store business data, including this application
 • E01 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx – row 42 – 2025 DR Test Scope = True; 2025 Backup/Restore DIV Scope = True
 • E02 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg – view 'Applications In Scope for DR Test BSI'
 • E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg – BIA results &amp; applications list review
@@ -4554,8 +4593,9 @@
       </c>
       <c r="R13" s="40" t="inlineStr">
         <is>
-          <t>[01 Management Attestation / In-Scope Applications]
+          <t xml:space="preserve">[01 Management Attestation / In-Scope Applications]
 MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png
+MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg
 [02 Business Line Approval Results – Email]
 BLA03 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf
 BLA04 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx
@@ -4570,7 +4610,8 @@
 E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg
 E07 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg
 E08 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg
-E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx
+</t>
         </is>
       </c>
       <c r="S13" s="42" t="inlineStr">
@@ -4879,9 +4920,10 @@
       </c>
       <c r="N14" s="69" t="inlineStr">
         <is>
-          <t>PASS – T24 is identified as in scope. The BCiC in-scope applications view (BSI In-Scope Applications-2026) shows App ID 1937 selected among the 10 applications flagged 2025 Backup/Restore DIV Scope = True; corroborated by the BCiC DR-scope export, the IT BIA/applications review and the management attestation.
+          <t>PASS – T24 is identified as in scope. The BCiC in-scope applications view BSI In-Scope Applications-2026 (MA01, Management_Attestation folder) shows App ID 1937 selected among the 10 applications flagged 2025 Backup/Restore DIV Scope = True, and the signed Management Attestation (MA02, §2) lists it among the 13 in-scope applications that store business data; corroborated by the BCiC DR-scope export (E01, E02), the IT BIA/applications review (E05) and the signed attestations (MA02, DMA02).
 Evidence location (BSI.IT.6.C7.3-Evidences):
 • MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png – BSI In-Scope Applications-2026 – App ID 1937 selected; 2025 DR Test Scope, 2025 Backup/Restore Test Scope and 2025 Backup/Restore DIV Scope = True
+• MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg – Management Attestation email 08/18/2026 – attached signed attestation (4069_001.pdf) §2 lists the 13 in-scope applications that store business data, including this application
 • E01 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx – row 43 – 2025 DR Test Scope = True; 2025 Backup/Restore DIV Scope = True
 • E02 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg – view 'Applications In Scope for DR Test BSI'
 • E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg – BIA results &amp; applications list review
@@ -4937,8 +4979,9 @@
       </c>
       <c r="R14" s="43" t="inlineStr">
         <is>
-          <t>[01 Management Attestation / In-Scope Applications]
+          <t xml:space="preserve">[01 Management Attestation / In-Scope Applications]
 MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png
+MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg
 [02 Business Line Approval Results – Email]
 BLA01 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf
 BLA02 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf
@@ -4969,7 +5012,8 @@
 E08 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg
 E09 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg
 E10 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg
-E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx
+</t>
         </is>
       </c>
       <c r="S14" s="42" t="inlineStr">
@@ -5469,7 +5513,7 @@
       <c r="R29" s="82" t="n"/>
       <c r="S29" s="82" t="n"/>
     </row>
-    <row r="30" ht="54" customHeight="1" s="71">
+    <row r="30" ht="42" customHeight="1" s="71">
       <c r="A30" s="86" t="inlineStr">
         <is>
           <t>BLA01</t>
@@ -5514,7 +5558,7 @@
       <c r="R30" s="82" t="n"/>
       <c r="S30" s="82" t="n"/>
     </row>
-    <row r="31" ht="54" customHeight="1" s="71">
+    <row r="31" ht="42" customHeight="1" s="71">
       <c r="A31" s="86" t="inlineStr">
         <is>
           <t>BLA02</t>
@@ -5559,7 +5603,7 @@
       <c r="R31" s="82" t="n"/>
       <c r="S31" s="82" t="n"/>
     </row>
-    <row r="32" ht="54" customHeight="1" s="71">
+    <row r="32" ht="42" customHeight="1" s="71">
       <c r="A32" s="86" t="inlineStr">
         <is>
           <t>BLA03</t>
@@ -5604,7 +5648,7 @@
       <c r="R32" s="82" t="n"/>
       <c r="S32" s="82" t="n"/>
     </row>
-    <row r="33" ht="54" customHeight="1" s="71">
+    <row r="33" ht="42" customHeight="1" s="71">
       <c r="A33" s="86" t="inlineStr">
         <is>
           <t>BLA04</t>
@@ -5649,7 +5693,7 @@
       <c r="R33" s="82" t="n"/>
       <c r="S33" s="82" t="n"/>
     </row>
-    <row r="34" ht="42" customHeight="1" s="71">
+    <row r="34" ht="30" customHeight="1" s="71">
       <c r="A34" s="86" t="inlineStr">
         <is>
           <t>BLA05</t>
@@ -5694,7 +5738,7 @@
       <c r="R34" s="82" t="n"/>
       <c r="S34" s="82" t="n"/>
     </row>
-    <row r="35" ht="42" customHeight="1" s="71">
+    <row r="35" ht="30" customHeight="1" s="71">
       <c r="A35" s="86" t="inlineStr">
         <is>
           <t>BLA06</t>
@@ -5819,7 +5863,7 @@
       <c r="R38" s="82" t="n"/>
       <c r="S38" s="82" t="n"/>
     </row>
-    <row r="39" ht="42" customHeight="1" s="71">
+    <row r="39" ht="30" customHeight="1" s="71">
       <c r="A39" s="86" t="inlineStr">
         <is>
           <t>DMA01</t>
@@ -5864,7 +5908,7 @@
       <c r="R39" s="82" t="n"/>
       <c r="S39" s="82" t="n"/>
     </row>
-    <row r="40" ht="90" customHeight="1" s="71">
+    <row r="40" ht="66" customHeight="1" s="71">
       <c r="A40" s="86" t="inlineStr">
         <is>
           <t>DMA02</t>
@@ -5909,7 +5953,7 @@
       <c r="R40" s="82" t="n"/>
       <c r="S40" s="82" t="n"/>
     </row>
-    <row r="41" ht="42" customHeight="1" s="71">
+    <row r="41" ht="30" customHeight="1" s="71">
       <c r="A41" s="86" t="inlineStr">
         <is>
           <t>DMA03</t>
@@ -5954,7 +5998,7 @@
       <c r="R41" s="82" t="n"/>
       <c r="S41" s="82" t="n"/>
     </row>
-    <row r="42" ht="42" customHeight="1" s="71">
+    <row r="42" ht="30" customHeight="1" s="71">
       <c r="A42" s="86" t="inlineStr">
         <is>
           <t>DMA04</t>
@@ -5999,7 +6043,7 @@
       <c r="R42" s="82" t="n"/>
       <c r="S42" s="82" t="n"/>
     </row>
-    <row r="43" ht="54" customHeight="1" s="71">
+    <row r="43" ht="42" customHeight="1" s="71">
       <c r="A43" s="86" t="inlineStr">
         <is>
           <t>DMA05</t>
@@ -6044,7 +6088,7 @@
       <c r="R43" s="82" t="n"/>
       <c r="S43" s="82" t="n"/>
     </row>
-    <row r="44" ht="54" customHeight="1" s="71">
+    <row r="44" ht="42" customHeight="1" s="71">
       <c r="A44" s="86" t="inlineStr">
         <is>
           <t>DMA06</t>
@@ -6089,7 +6133,7 @@
       <c r="R44" s="82" t="n"/>
       <c r="S44" s="82" t="n"/>
     </row>
-    <row r="45" ht="42" customHeight="1" s="71">
+    <row r="45" ht="30" customHeight="1" s="71">
       <c r="A45" s="86" t="inlineStr">
         <is>
           <t>DMA07</t>
@@ -6134,7 +6178,7 @@
       <c r="R45" s="82" t="n"/>
       <c r="S45" s="82" t="n"/>
     </row>
-    <row r="46" ht="42" customHeight="1" s="71">
+    <row r="46" ht="30" customHeight="1" s="71">
       <c r="A46" s="86" t="inlineStr">
         <is>
           <t>DMA08</t>
@@ -6179,7 +6223,7 @@
       <c r="R46" s="82" t="n"/>
       <c r="S46" s="82" t="n"/>
     </row>
-    <row r="47" ht="42" customHeight="1" s="71">
+    <row r="47" ht="30" customHeight="1" s="71">
       <c r="A47" s="86" t="inlineStr">
         <is>
           <t>DMA09</t>
@@ -6224,7 +6268,7 @@
       <c r="R47" s="82" t="n"/>
       <c r="S47" s="82" t="n"/>
     </row>
-    <row r="48" ht="42" customHeight="1" s="71">
+    <row r="48" ht="30" customHeight="1" s="71">
       <c r="A48" s="86" t="inlineStr">
         <is>
           <t>DMA10</t>
@@ -6269,7 +6313,7 @@
       <c r="R48" s="82" t="n"/>
       <c r="S48" s="82" t="n"/>
     </row>
-    <row r="49" ht="42" customHeight="1" s="71">
+    <row r="49" ht="30" customHeight="1" s="71">
       <c r="A49" s="86" t="inlineStr">
         <is>
           <t>DMA11</t>
@@ -6314,7 +6358,7 @@
       <c r="R49" s="82" t="n"/>
       <c r="S49" s="82" t="n"/>
     </row>
-    <row r="50" ht="42" customHeight="1" s="71">
+    <row r="50" ht="30" customHeight="1" s="71">
       <c r="A50" s="86" t="inlineStr">
         <is>
           <t>DMA12</t>
@@ -6359,7 +6403,7 @@
       <c r="R50" s="82" t="n"/>
       <c r="S50" s="82" t="n"/>
     </row>
-    <row r="51" ht="42" customHeight="1" s="71">
+    <row r="51" ht="30" customHeight="1" s="71">
       <c r="A51" s="86" t="inlineStr">
         <is>
           <t>DMA13</t>
@@ -6484,7 +6528,7 @@
       <c r="R54" s="82" t="n"/>
       <c r="S54" s="82" t="n"/>
     </row>
-    <row r="55" ht="66" customHeight="1" s="71">
+    <row r="55" ht="42" customHeight="1" s="71">
       <c r="A55" s="86" t="inlineStr">
         <is>
           <t>MA01</t>
@@ -6529,35 +6573,35 @@
       <c r="R55" s="82" t="n"/>
       <c r="S55" s="82" t="n"/>
     </row>
-    <row r="56" ht="30" customHeight="1" s="71">
+    <row r="56" ht="78" customHeight="1" s="71">
       <c r="A56" s="86" t="inlineStr">
         <is>
-          <t>E01</t>
+          <t>MA02</t>
         </is>
       </c>
       <c r="B56" s="86" t="inlineStr">
         <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx</t>
+          <t>BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg</t>
         </is>
       </c>
       <c r="C56" s="86" t="inlineStr">
         <is>
-          <t>BCiC – Applications In Scope for DR Test BSI</t>
+          <t>08/18/2026 – Frank Puentes</t>
         </is>
       </c>
       <c r="D56" s="86" t="inlineStr">
         <is>
-          <t>BCiC export</t>
+          <t>Email + signed management attestation</t>
         </is>
       </c>
       <c r="E56" s="86" t="inlineStr">
         <is>
-          <t>BCiC export of the BSI DR-scope population (43 applications) with Exercise Date and 2025 DR / Backup-Restore / DIV scope flags.</t>
+          <t>Management Attestation email: Frank Puentes (Executive Director, Payments &amp; Cash Management) returns the signed attestation (attachment 4069_001.pdf) to Cesar Vidal. The quoted Cesar Vidal request (08/17/2026) confirms the DR exercises of 11/15/2025 and 02/21/2026 and attaches the BCiC DIV export; the signed attestation §2 lists the 13 in-scope BSI applications that store business data, including all 10 tested applications. Filed in the Management_Attestation folder as received; the same message is also filed as DMA03 for the business line approval attribute.</t>
         </is>
       </c>
       <c r="F56" s="86" t="inlineStr">
         <is>
-          <t>Samples: 1822, 1867, 1868, 3299, 4052, 3301, 1903, 1917, 1936, 1937; columns: B, C, D, K, L, N</t>
+          <t>Samples: 1822, 1867, 1868, 3299, 4052, 3301, 1903, 1917, 1936, 1937; columns: N</t>
         </is>
       </c>
       <c r="G56" s="82" t="n"/>
@@ -6577,32 +6621,32 @@
     <row r="57" ht="30" customHeight="1" s="71">
       <c r="A57" s="86" t="inlineStr">
         <is>
-          <t>E02</t>
+          <t>E01</t>
         </is>
       </c>
       <c r="B57" s="86" t="inlineStr">
         <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg</t>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx</t>
         </is>
       </c>
       <c r="C57" s="86" t="inlineStr">
         <is>
-          <t>09/10/2026 – Cesar Vidal</t>
+          <t>BCiC – Applications In Scope for DR Test BSI</t>
         </is>
       </c>
       <c r="D57" s="86" t="inlineStr">
         <is>
-          <t>BCiC screenshot</t>
+          <t>BCiC export</t>
         </is>
       </c>
       <c r="E57" s="86" t="inlineStr">
         <is>
-          <t>BCiC Applications screen with view 'Applications In Scope for DR Test BSI' selected (1–20 of 43 items).</t>
+          <t>BCiC export of the BSI DR-scope population (43 applications) with Exercise Date and 2025 DR / Backup-Restore / DIV scope flags.</t>
         </is>
       </c>
       <c r="F57" s="86" t="inlineStr">
         <is>
-          <t>Samples: 1822, 1867, 1868, 3299, 4052, 3301, 1903, 1917, 1936, 1937; columns: D, K, N</t>
+          <t>Samples: 1822, 1867, 1868, 3299, 4052, 3301, 1903, 1917, 1936, 1937; columns: B, C, D, K, L, N</t>
         </is>
       </c>
       <c r="G57" s="82" t="n"/>
@@ -6619,35 +6663,35 @@
       <c r="R57" s="82" t="n"/>
       <c r="S57" s="82" t="n"/>
     </row>
-    <row r="58" ht="42" customHeight="1" s="71">
+    <row r="58" ht="30" customHeight="1" s="71">
       <c r="A58" s="86" t="inlineStr">
         <is>
-          <t>E03</t>
+          <t>E02</t>
         </is>
       </c>
       <c r="B58" s="86" t="inlineStr">
         <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg</t>
         </is>
       </c>
       <c r="C58" s="86" t="inlineStr">
         <is>
-          <t>BCiC – Data Integrity Validation Testing (62 records)</t>
+          <t>09/10/2026 – Cesar Vidal</t>
         </is>
       </c>
       <c r="D58" s="86" t="inlineStr">
         <is>
-          <t>BCiC export</t>
+          <t>BCiC screenshot</t>
         </is>
       </c>
       <c r="E58" s="86" t="inlineStr">
         <is>
-          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Y/N Format/Headers/Content, Attestation Date / Provided By. Row numbers quoted are Excel rows.</t>
+          <t>BCiC Applications screen with view 'Applications In Scope for DR Test BSI' selected (1–20 of 43 items).</t>
         </is>
       </c>
       <c r="F58" s="86" t="inlineStr">
         <is>
-          <t>Samples: 1822, 1867, 1868, 3299, 4052, 3301, 1903, 1917, 1936, 1937; columns: B, C, D, E, F, G, H, I, K, L, M, O, P</t>
+          <t>Samples: 1822, 1867, 1868, 3299, 4052, 3301, 1903, 1917, 1936, 1937; columns: D, K, N</t>
         </is>
       </c>
       <c r="G58" s="82" t="n"/>
@@ -6664,35 +6708,35 @@
       <c r="R58" s="82" t="n"/>
       <c r="S58" s="82" t="n"/>
     </row>
-    <row r="59" ht="42" customHeight="1" s="71">
+    <row r="59" ht="30" customHeight="1" s="71">
       <c r="A59" s="86" t="inlineStr">
         <is>
-          <t>E04</t>
+          <t>E03</t>
         </is>
       </c>
       <c r="B59" s="86" t="inlineStr">
         <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg</t>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
         </is>
       </c>
       <c r="C59" s="86" t="inlineStr">
         <is>
-          <t>09/10/2026 – Cesar Vidal</t>
+          <t>BCiC – Data Integrity Validation Testing (62 records)</t>
         </is>
       </c>
       <c r="D59" s="86" t="inlineStr">
         <is>
-          <t>BCiC screenshot</t>
+          <t>BCiC export</t>
         </is>
       </c>
       <c r="E59" s="86" t="inlineStr">
         <is>
-          <t>BCiC 'Data Integrity Validation Testing' screen (1–20 of 66 items) showing tester, validation date, manager, approval date, Y/N results and attestation fields.</t>
+          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Y/N Format/Headers/Content, Attestation Date / Provided By. Row numbers quoted are Excel rows.</t>
         </is>
       </c>
       <c r="F59" s="86" t="inlineStr">
         <is>
-          <t>Samples: 1822, 1867, 1868, 3299, 4052, 3301, 1903, 1917, 1936, 1937; columns: D, E, F, G, H, K, P</t>
+          <t>Samples: 1822, 1867, 1868, 3299, 4052, 3301, 1903, 1917, 1936, 1937; columns: B, C, D, E, F, G, H, I, K, L, M, O, P</t>
         </is>
       </c>
       <c r="G59" s="82" t="n"/>
@@ -6709,35 +6753,35 @@
       <c r="R59" s="82" t="n"/>
       <c r="S59" s="82" t="n"/>
     </row>
-    <row r="60" ht="42" customHeight="1" s="71">
+    <row r="60" ht="30" customHeight="1" s="71">
       <c r="A60" s="86" t="inlineStr">
         <is>
-          <t>E05</t>
+          <t>E04</t>
         </is>
       </c>
       <c r="B60" s="86" t="inlineStr">
         <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg</t>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg</t>
         </is>
       </c>
       <c r="C60" s="86" t="inlineStr">
         <is>
-          <t>09/15/2025 – Elizabeth Noda</t>
+          <t>09/10/2026 – Cesar Vidal</t>
         </is>
       </c>
       <c r="D60" s="86" t="inlineStr">
         <is>
-          <t>Meeting invite</t>
+          <t>BCiC screenshot</t>
         </is>
       </c>
       <c r="E60" s="86" t="inlineStr">
         <is>
-          <t>IT DR meeting invite to review the 2025 BIA results and applications list ahead of the DR exercise (same invite re-sent 09/18/2025 – duplicate E06 removed).</t>
+          <t>BCiC 'Data Integrity Validation Testing' screen (1–20 of 66 items) showing tester, validation date, manager, approval date, Y/N results and attestation fields.</t>
         </is>
       </c>
       <c r="F60" s="86" t="inlineStr">
         <is>
-          <t>Samples: 1822, 1867, 1868, 3299, 4052, 3301, 1903, 1917, 1936, 1937; columns: M, N</t>
+          <t>Samples: 1822, 1867, 1868, 3299, 4052, 3301, 1903, 1917, 1936, 1937; columns: D, E, F, G, H, K, P</t>
         </is>
       </c>
       <c r="G60" s="82" t="n"/>
@@ -6754,35 +6798,35 @@
       <c r="R60" s="82" t="n"/>
       <c r="S60" s="82" t="n"/>
     </row>
-    <row r="61" ht="126" customHeight="1" s="71">
+    <row r="61" ht="30" customHeight="1" s="71">
       <c r="A61" s="86" t="inlineStr">
         <is>
-          <t>E07</t>
+          <t>E05</t>
         </is>
       </c>
       <c r="B61" s="86" t="inlineStr">
         <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg</t>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg</t>
         </is>
       </c>
       <c r="C61" s="86" t="inlineStr">
         <is>
-          <t>11/15/2025 – Frank Puentes</t>
+          <t>09/15/2025 – Elizabeth Noda</t>
         </is>
       </c>
       <c r="D61" s="86" t="inlineStr">
         <is>
-          <t>Email + report attachments</t>
+          <t>Meeting invite</t>
         </is>
       </c>
       <c r="E61" s="86" t="inlineStr">
         <is>
-          <t>Pre-DR (11/14/2025) source reports: Fedlink, OFAC ACH/FED/SWIFT, Payment Monitor, SWIFT Interface Monitor, outgoing Fedwire/SWIFT. Embedded attachments: FEDLINK INCOMING FEDWIRES 111425 0523PM.pdf; FEDLINK OUTGOING FEDWIRES 111425 0523PM.pdf; OFAC ACH 111425 0512PM.pdf; OFAC FED 111425 0511PM.pdf; OFAC SWIFT 111425 0511PM.pdf; OUTGOING FEDWIRE 111425 506PM.xls; OUTGOING SWIFT 111425 509PM.xls; PAYMENT MONITOR INCOMING FEDWIRE 111425 516PM PG1.pdf; PAYMENT MONITOR INCOMING FEDWIRE 111425 516PM PG2.pdf; PAYMENT MONITOR OUTGOING FEDWIRE 111425 516PM PG1.pdf; PAYMENT MONITOR OUTGOING FEDWIRE 111425 516PM PG2.pdf; SWIFT INTERFACE MONITOR 111425 519PM.pdf; SWIFT INTERFACE MONITOR 111425 520PM 2ND SAMPLE.pdf.</t>
+          <t>IT DR meeting invite to review the 2025 BIA results and applications list ahead of the DR exercise (same invite re-sent 09/18/2025 – duplicate E06 removed).</t>
         </is>
       </c>
       <c r="F61" s="86" t="inlineStr">
         <is>
-          <t>Samples: 3301, 1903, 1936, 1937; columns: F</t>
+          <t>Samples: 1822, 1867, 1868, 3299, 4052, 3301, 1903, 1917, 1936, 1937; columns: M, N</t>
         </is>
       </c>
       <c r="G61" s="82" t="n"/>
@@ -6799,15 +6843,15 @@
       <c r="R61" s="82" t="n"/>
       <c r="S61" s="82" t="n"/>
     </row>
-    <row r="62" ht="126" customHeight="1" s="71">
+    <row r="62" ht="90" customHeight="1" s="71">
       <c r="A62" s="86" t="inlineStr">
         <is>
-          <t>E08</t>
+          <t>E07</t>
         </is>
       </c>
       <c r="B62" s="86" t="inlineStr">
         <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg</t>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg</t>
         </is>
       </c>
       <c r="C62" s="86" t="inlineStr">
@@ -6822,12 +6866,12 @@
       </c>
       <c r="E62" s="86" t="inlineStr">
         <is>
-          <t>DR test-day (11/15/2025) re-run of the same reports for comparison with 11/14/2025 source. Embedded attachments: FEDLINK INCOMING FEDWIRES 111425 -1115 1148AM.pdf; FEDLINK OUTGOINT TRANSFERS 114125 - 111525 1144AM.pdf; OFAC ACH 111425 - 11152025 1126AM.pdf; OFAC FED 111425 - 111525 1126AM.pdf; OFAC SWIFT 111425 - 111525 1128AM.pdf; OUTGOING FEDWIRE 111525 1025AM.xls; OUTGOING SWIFT 111525 1026AM.xls; PAYMENT MONITOR 111424 - 111525 PG 11156AM.pdf; PAYMENT MONITOR 111425 - 111525 PG 2 1158AM.pdf; PAYMENT MONITOR OUTGOING 111425 - 111525 PG 1 1156AM.pdf; PAYMENT MONITOR OUTGOING 111425 - 111525 PG 2 1156AM.pdf; SWIFT INTERFACE MONITOR INCOMING MT103 111425 - 111525 1152AM.pdf; SWIFT INTERFACE MONITOR INCOMING MT199 111425 -111525 1152AM.pdf.</t>
+          <t>Pre-DR (11/14/2025) source reports: Fedlink, OFAC ACH/FED/SWIFT, Payment Monitor, SWIFT Interface Monitor, outgoing Fedwire/SWIFT. Embedded attachments: FEDLINK INCOMING FEDWIRES 111425 0523PM.pdf; FEDLINK OUTGOING FEDWIRES 111425 0523PM.pdf; OFAC ACH 111425 0512PM.pdf; OFAC FED 111425 0511PM.pdf; OFAC SWIFT 111425 0511PM.pdf; OUTGOING FEDWIRE 111425 506PM.xls; OUTGOING SWIFT 111425 509PM.xls; PAYMENT MONITOR INCOMING FEDWIRE 111425 516PM PG1.pdf; PAYMENT MONITOR INCOMING FEDWIRE 111425 516PM PG2.pdf; PAYMENT MONITOR OUTGOING FEDWIRE 111425 516PM PG1.pdf; PAYMENT MONITOR OUTGOING FEDWIRE 111425 516PM PG2.pdf; SWIFT INTERFACE MONITOR 111425 519PM.pdf; SWIFT INTERFACE MONITOR 111425 520PM 2ND SAMPLE.pdf.</t>
         </is>
       </c>
       <c r="F62" s="86" t="inlineStr">
         <is>
-          <t>Samples: 3301, 1903, 1936, 1937; columns: F, M</t>
+          <t>Samples: 3301, 1903, 1936, 1937; columns: F</t>
         </is>
       </c>
       <c r="G62" s="82" t="n"/>
@@ -6844,35 +6888,35 @@
       <c r="R62" s="82" t="n"/>
       <c r="S62" s="82" t="n"/>
     </row>
-    <row r="63" ht="54" customHeight="1" s="71">
+    <row r="63" ht="90" customHeight="1" s="71">
       <c r="A63" s="86" t="inlineStr">
         <is>
-          <t>E09</t>
+          <t>E08</t>
         </is>
       </c>
       <c r="B63" s="86" t="inlineStr">
         <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg</t>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg</t>
         </is>
       </c>
       <c r="C63" s="86" t="inlineStr">
         <is>
-          <t>03/03/2026 – 05/05/2026 – Claudia Romero</t>
+          <t>11/15/2025 – Frank Puentes</t>
         </is>
       </c>
       <c r="D63" s="86" t="inlineStr">
         <is>
-          <t>Email approval</t>
+          <t>Email + report attachments</t>
         </is>
       </c>
       <c r="E63" s="86" t="inlineStr">
         <is>
-          <t>Client Back Office test evidence (Mariorly Morales, Ilumel Rodriguez, Rolando Bonilla) and Claudia Romero "Approved." 05/05/2026. Thread maps ACH Express, FedExport, FedImport, Imaging101 to Client Back Office / Claudia Romero.</t>
+          <t>DR test-day (11/15/2025) re-run of the same reports for comparison with 11/14/2025 source. Embedded attachments: FEDLINK INCOMING FEDWIRES 111425 -1115 1148AM.pdf; FEDLINK OUTGOINT TRANSFERS 114125 - 111525 1144AM.pdf; OFAC ACH 111425 - 11152025 1126AM.pdf; OFAC FED 111425 - 111525 1126AM.pdf; OFAC SWIFT 111425 - 111525 1128AM.pdf; OUTGOING FEDWIRE 111525 1025AM.xls; OUTGOING SWIFT 111525 1026AM.xls; PAYMENT MONITOR 111424 - 111525 PG 11156AM.pdf; PAYMENT MONITOR 111425 - 111525 PG 2 1158AM.pdf; PAYMENT MONITOR OUTGOING 111425 - 111525 PG 1 1156AM.pdf; PAYMENT MONITOR OUTGOING 111425 - 111525 PG 2 1156AM.pdf; SWIFT INTERFACE MONITOR INCOMING MT103 111425 - 111525 1152AM.pdf; SWIFT INTERFACE MONITOR INCOMING MT199 111425 -111525 1152AM.pdf.</t>
         </is>
       </c>
       <c r="F63" s="86" t="inlineStr">
         <is>
-          <t>Samples: 1822, 1867, 1868, 3299, 1937; columns: E, G, H, J, M, N, O</t>
+          <t>Samples: 3301, 1903, 1936, 1937; columns: F, M</t>
         </is>
       </c>
       <c r="G63" s="82" t="n"/>
@@ -6892,17 +6936,17 @@
     <row r="64" ht="42" customHeight="1" s="71">
       <c r="A64" s="86" t="inlineStr">
         <is>
-          <t>E10</t>
+          <t>E09</t>
         </is>
       </c>
       <c r="B64" s="86" t="inlineStr">
         <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg</t>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg</t>
         </is>
       </c>
       <c r="C64" s="86" t="inlineStr">
         <is>
-          <t>03/09/2026 – Lina Acuna</t>
+          <t>03/03/2026 – 05/05/2026 – Claudia Romero</t>
         </is>
       </c>
       <c r="D64" s="86" t="inlineStr">
@@ -6912,12 +6956,12 @@
       </c>
       <c r="E64" s="86" t="inlineStr">
         <is>
-          <t>Finance DIV results chart (Jose Acero) and Lina Acuna "Approved" 03/09/2026 (T24 / ReconXpert backup-restore).</t>
+          <t>Client Back Office test evidence (Mariorly Morales, Ilumel Rodriguez, Rolando Bonilla) and Claudia Romero "Approved." 05/05/2026. Thread maps ACH Express, FedExport, FedImport, Imaging101 to Client Back Office / Claudia Romero.</t>
         </is>
       </c>
       <c r="F64" s="86" t="inlineStr">
         <is>
-          <t>Samples: 1917, 1937; columns: M</t>
+          <t>Samples: 1822, 1867, 1868, 3299, 1937; columns: E, G, H, J, M, N, O</t>
         </is>
       </c>
       <c r="G64" s="82" t="n"/>
@@ -6934,35 +6978,35 @@
       <c r="R64" s="82" t="n"/>
       <c r="S64" s="82" t="n"/>
     </row>
-    <row r="65" ht="42" customHeight="1" s="71">
+    <row r="65" ht="30" customHeight="1" s="71">
       <c r="A65" s="86" t="inlineStr">
         <is>
-          <t>E13</t>
+          <t>E10</t>
         </is>
       </c>
       <c r="B65" s="86" t="inlineStr">
         <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg</t>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg</t>
         </is>
       </c>
       <c r="C65" s="86" t="inlineStr">
         <is>
-          <t>11/13/2024 – T24 backup user</t>
+          <t>03/09/2026 – Lina Acuna</t>
         </is>
       </c>
       <c r="D65" s="86" t="inlineStr">
         <is>
-          <t>System email</t>
+          <t>Email approval</t>
         </is>
       </c>
       <c r="E65" s="86" t="inlineStr">
         <is>
-          <t>T24 environment refresh log – prior period (outside review period); supplemental only.</t>
+          <t>Finance DIV results chart (Jose Acero) and Lina Acuna "Approved" 03/09/2026 (T24 / ReconXpert backup-restore).</t>
         </is>
       </c>
       <c r="F65" s="86" t="inlineStr">
         <is>
-          <t>Samples: —; columns: — (supplemental)</t>
+          <t>Samples: 1917, 1937; columns: M</t>
         </is>
       </c>
       <c r="G65" s="82" t="n"/>
@@ -6979,35 +7023,35 @@
       <c r="R65" s="82" t="n"/>
       <c r="S65" s="82" t="n"/>
     </row>
-    <row r="66" ht="42" customHeight="1" s="71">
+    <row r="66" ht="30" customHeight="1" s="71">
       <c r="A66" s="86" t="inlineStr">
         <is>
-          <t>E16b</t>
+          <t>E13</t>
         </is>
       </c>
       <c r="B66" s="86" t="inlineStr">
         <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg</t>
         </is>
       </c>
       <c r="C66" s="86" t="inlineStr">
         <is>
-          <t>08/2026 – BCiC export sent with attestation request</t>
+          <t>11/13/2024 – T24 backup user</t>
         </is>
       </c>
       <c r="D66" s="86" t="inlineStr">
         <is>
-          <t>BCiC export</t>
+          <t>System email</t>
         </is>
       </c>
       <c r="E66" s="86" t="inlineStr">
         <is>
-          <t>BCiC DIV export 2025-26 (64 rows; no manager columns) sent to managers with the attestation request and returned by M. T. Del Cerro (DMA05). Row numbers are Excel rows.</t>
+          <t>T24 environment refresh log – prior period (outside review period); supplemental only.</t>
         </is>
       </c>
       <c r="F66" s="86" t="inlineStr">
         <is>
-          <t>Samples: 1822, 1867, 1868, 3299, 4052, 3301, 1903, 1917, 1936, 1937; columns: B, D, E, F, I, K, P</t>
+          <t>Samples: —; columns: — (supplemental)</t>
         </is>
       </c>
       <c r="G66" s="82" t="n"/>
@@ -7024,13 +7068,37 @@
       <c r="R66" s="82" t="n"/>
       <c r="S66" s="82" t="n"/>
     </row>
-    <row r="67" s="71">
-      <c r="A67" s="82" t="n"/>
-      <c r="B67" s="82" t="n"/>
-      <c r="C67" s="82" t="n"/>
-      <c r="D67" s="82" t="n"/>
-      <c r="E67" s="82" t="n"/>
-      <c r="F67" s="82" t="n"/>
+    <row r="67" ht="30" customHeight="1" s="71">
+      <c r="A67" s="86" t="inlineStr">
+        <is>
+          <t>E16b</t>
+        </is>
+      </c>
+      <c r="B67" s="86" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+        </is>
+      </c>
+      <c r="C67" s="86" t="inlineStr">
+        <is>
+          <t>08/2026 – BCiC export sent with attestation request</t>
+        </is>
+      </c>
+      <c r="D67" s="86" t="inlineStr">
+        <is>
+          <t>BCiC export</t>
+        </is>
+      </c>
+      <c r="E67" s="86" t="inlineStr">
+        <is>
+          <t>BCiC DIV export 2025-26 (64 rows; no manager columns) sent to managers with the attestation request and returned by M. T. Del Cerro (DMA05). Row numbers are Excel rows.</t>
+        </is>
+      </c>
+      <c r="F67" s="86" t="inlineStr">
+        <is>
+          <t>Samples: 1822, 1867, 1868, 3299, 4052, 3301, 1903, 1917, 1936, 1937; columns: B, D, E, F, I, K, P</t>
+        </is>
+      </c>
       <c r="G67" s="82" t="n"/>
       <c r="H67" s="82" t="n"/>
       <c r="I67" s="82" t="n"/>
@@ -7045,12 +7113,19 @@
       <c r="R67" s="82" t="n"/>
       <c r="S67" s="82" t="n"/>
     </row>
-    <row r="68" ht="22" customHeight="1" s="71">
-      <c r="A68" s="73" t="inlineStr">
-        <is>
-          <t>Observations for reviewer consideration (do not change the PASS conclusions unless the reviewer determines otherwise)</t>
-        </is>
-      </c>
+    <row r="68" s="71">
+      <c r="A68" s="82" t="n"/>
+      <c r="B68" s="82" t="n"/>
+      <c r="C68" s="82" t="n"/>
+      <c r="D68" s="82" t="n"/>
+      <c r="E68" s="82" t="n"/>
+      <c r="F68" s="82" t="n"/>
+      <c r="G68" s="82" t="n"/>
+      <c r="H68" s="82" t="n"/>
+      <c r="I68" s="82" t="n"/>
+      <c r="J68" s="82" t="n"/>
+      <c r="K68" s="82" t="n"/>
+      <c r="L68" s="82" t="n"/>
       <c r="M68" s="82" t="n"/>
       <c r="N68" s="82" t="n"/>
       <c r="O68" s="82" t="n"/>
@@ -7059,39 +7134,12 @@
       <c r="R68" s="82" t="n"/>
       <c r="S68" s="82" t="n"/>
     </row>
-    <row r="69" ht="30" customHeight="1" s="71">
-      <c r="A69" s="85" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B69" s="85" t="inlineStr">
-        <is>
-          <t>Observation</t>
-        </is>
-      </c>
-      <c r="C69" s="85" t="inlineStr">
-        <is>
-          <t>Samples affected</t>
-        </is>
-      </c>
-      <c r="D69" s="85" t="inlineStr">
-        <is>
-          <t>Evidence</t>
-        </is>
-      </c>
-      <c r="E69" s="85" t="inlineStr">
-        <is>
-          <t>Impact / reviewer consideration</t>
-        </is>
-      </c>
-      <c r="F69" s="85" t="inlineStr"/>
-      <c r="G69" s="82" t="n"/>
-      <c r="H69" s="82" t="n"/>
-      <c r="I69" s="82" t="n"/>
-      <c r="J69" s="82" t="n"/>
-      <c r="K69" s="82" t="n"/>
-      <c r="L69" s="82" t="n"/>
+    <row r="69" ht="22" customHeight="1" s="71">
+      <c r="A69" s="73" t="inlineStr">
+        <is>
+          <t>Observations for reviewer consideration (do not change the PASS conclusions unless the reviewer determines otherwise)</t>
+        </is>
+      </c>
       <c r="M69" s="82" t="n"/>
       <c r="N69" s="82" t="n"/>
       <c r="O69" s="82" t="n"/>
@@ -7100,31 +7148,33 @@
       <c r="R69" s="82" t="n"/>
       <c r="S69" s="82" t="n"/>
     </row>
-    <row r="70" ht="90" customHeight="1" s="71">
-      <c r="A70" s="87" t="n">
-        <v>1</v>
-      </c>
-      <c r="B70" s="87" t="inlineStr">
-        <is>
-          <t>Business line approvals for 33 of 56 in-scope DIV records were obtained through retrospective management attestations dated 08/17/2026 – 09/09/2026, i.e. after the review period end (06/01/2026) and ~9-10 months after the 11/15/2025 DIV testing. A further 13 records (BSA/AML/OFAC and Payments) carry in-period BCiC approval dates (11/15/2025, 12/18/2025) supported only by 08/2026 signed attestations. 10 records have in-period approval emails (E09, BLA06).</t>
-        </is>
-      </c>
-      <c r="C70" s="87" t="inlineStr">
-        <is>
-          <t>3299, 4052, 3301, 1903, 1936, 1937</t>
-        </is>
-      </c>
-      <c r="D70" s="87" t="inlineStr">
-        <is>
-          <t>Folder 03 (DMA01–DMA12); E03 approval dates</t>
-        </is>
-      </c>
-      <c r="E70" s="87" t="inlineStr">
-        <is>
-          <t>Approval is evidenced for 100% of records; timing is an observation. The attestation (DMA02 attachment §3.6) commits to contemporaneous approval going forward. Reviewer to conclude whether retrospective approval satisfies the control for the period.</t>
-        </is>
-      </c>
-      <c r="F70" s="87" t="inlineStr"/>
+    <row r="70" ht="30" customHeight="1" s="71">
+      <c r="A70" s="85" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B70" s="85" t="inlineStr">
+        <is>
+          <t>Observation</t>
+        </is>
+      </c>
+      <c r="C70" s="85" t="inlineStr">
+        <is>
+          <t>Samples affected</t>
+        </is>
+      </c>
+      <c r="D70" s="85" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="E70" s="85" t="inlineStr">
+        <is>
+          <t>Impact / reviewer consideration</t>
+        </is>
+      </c>
+      <c r="F70" s="85" t="inlineStr"/>
       <c r="G70" s="82" t="n"/>
       <c r="H70" s="82" t="n"/>
       <c r="I70" s="82" t="n"/>
@@ -7139,28 +7189,28 @@
       <c r="R70" s="82" t="n"/>
       <c r="S70" s="82" t="n"/>
     </row>
-    <row r="71" ht="78" customHeight="1" s="71">
+    <row r="71" ht="66" customHeight="1" s="71">
       <c r="A71" s="87" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B71" s="87" t="inlineStr">
         <is>
-          <t>Self-approval: the business tester and the approving Department Manager are the same person for BSA/AML/OFAC (David Marquez), Payments (Franklin Puentes), Investment Operations (Michelle Oropesa), Treasury (Martha Sullivan), Digital Wealth (Victoria Fernandez), Client Servicing Unit (Liliana Vizhnay), Commercial Middle Office (Miguel Orozco – Imaging101 / T24 row 15, 51) and Financial Analysis (Sadis Alvarenga).</t>
+          <t>Business line approvals for 33 of 56 in-scope DIV records were obtained through retrospective management attestations dated 08/17/2026 – 09/09/2026, i.e. after the review period end (06/01/2026) and ~9-10 months after the 11/15/2025 DIV testing. A further 13 records (BSA/AML/OFAC and Payments) carry in-period BCiC approval dates (11/15/2025, 12/18/2025) supported only by 08/2026 signed attestations. 10 records have in-period approval emails (E09, BLA06).</t>
         </is>
       </c>
       <c r="C71" s="87" t="inlineStr">
         <is>
-          <t>3299, 4052, 3301, 1903, 1917, 1936, 1937</t>
+          <t>3299, 4052, 3301, 1903, 1936, 1937</t>
         </is>
       </c>
       <c r="D71" s="87" t="inlineStr">
         <is>
-          <t>E03 tester vs manager columns</t>
+          <t>Folder 03 (DMA01–DMA12); E03 approval dates</t>
         </is>
       </c>
       <c r="E71" s="87" t="inlineStr">
         <is>
-          <t>Segregation-of-duties observation; the approvers are the business line heads for those areas.</t>
+          <t>Approval is evidenced for 100% of records; timing is an observation. The attestation (DMA02 attachment §3.6) commits to contemporaneous approval going forward. Reviewer to conclude whether retrospective approval satisfies the control for the period.</t>
         </is>
       </c>
       <c r="F71" s="87" t="inlineStr"/>
@@ -7178,28 +7228,28 @@
       <c r="R71" s="82" t="n"/>
       <c r="S71" s="82" t="n"/>
     </row>
-    <row r="72" ht="30" customHeight="1" s="71">
+    <row r="72" ht="54" customHeight="1" s="71">
       <c r="A72" s="87" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B72" s="87" t="inlineStr">
         <is>
-          <t>FedExport – BCiC Department Manager Approval Date 06/05/2026 (E03 row 9, E04) vs Claudia Romero "Approved." 05/05/2026 (E09).</t>
+          <t>Self-approval: the business tester and the approving Department Manager are the same person for BSA/AML/OFAC (David Marquez), Payments (Franklin Puentes), Investment Operations (Michelle Oropesa), Treasury (Martha Sullivan), Digital Wealth (Victoria Fernandez), Client Servicing Unit (Liliana Vizhnay), Commercial Middle Office (Miguel Orozco – Imaging101 / T24 row 15, 51) and Financial Analysis (Sadis Alvarenga).</t>
         </is>
       </c>
       <c r="C72" s="87" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>3299, 4052, 3301, 1903, 1917, 1936, 1937</t>
         </is>
       </c>
       <c r="D72" s="87" t="inlineStr">
         <is>
-          <t>E03, E04, E09</t>
+          <t>E03 tester vs manager columns</t>
         </is>
       </c>
       <c r="E72" s="87" t="inlineStr">
         <is>
-          <t>Likely BCiC data-entry error; recommend management correct the BCiC record.</t>
+          <t>Segregation-of-duties observation; the approvers are the business line heads for those areas.</t>
         </is>
       </c>
       <c r="F72" s="87" t="inlineStr"/>
@@ -7219,26 +7269,26 @@
     </row>
     <row r="73" ht="30" customHeight="1" s="71">
       <c r="A73" s="87" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B73" s="87" t="inlineStr">
         <is>
-          <t>BLA02 (BSA/AML/OFAC) test script – DIV Yes/No answer boxes are blank.</t>
+          <t>FedExport – BCiC Department Manager Approval Date 06/05/2026 (E03 row 9, E04) vs Claudia Romero "Approved." 05/05/2026 (E09).</t>
         </is>
       </c>
       <c r="C73" s="87" t="inlineStr">
         <is>
-          <t>3299, 1903, 1936, 1937</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="D73" s="87" t="inlineStr">
         <is>
-          <t>BLA02 p.1</t>
+          <t>E03, E04, E09</t>
         </is>
       </c>
       <c r="E73" s="87" t="inlineStr">
         <is>
-          <t>Mitigated by production vs test-day screenshots in BLA02, BCiC Y/Y/Y (E03) and signed attestation (DMA02 attachment).</t>
+          <t>Likely BCiC data-entry error; recommend management correct the BCiC record.</t>
         </is>
       </c>
       <c r="F73" s="87" t="inlineStr"/>
@@ -7256,28 +7306,28 @@
       <c r="R73" s="82" t="n"/>
       <c r="S73" s="82" t="n"/>
     </row>
-    <row r="74" ht="54" customHeight="1" s="71">
+    <row r="74" ht="30" customHeight="1" s="71">
       <c r="A74" s="87" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B74" s="87" t="inlineStr">
         <is>
-          <t>BSA T24 record (E03 row 8) Attestation Date 08/29/2026 vs signed attestation 8/19/2026 (DMA02 attachment); Financial Risk manager recorded as "Xavier Caisapanta" in BCiC while the approval email is from Ivan Caisapanta (DMA08).</t>
+          <t>BLA02 (BSA/AML/OFAC) test script – DIV Yes/No answer boxes are blank.</t>
         </is>
       </c>
       <c r="C74" s="87" t="inlineStr">
         <is>
-          <t>1937</t>
+          <t>3299, 1903, 1936, 1937</t>
         </is>
       </c>
       <c r="D74" s="87" t="inlineStr">
         <is>
-          <t>E03, DMA02, DMA08</t>
+          <t>BLA02 p.1</t>
         </is>
       </c>
       <c r="E74" s="87" t="inlineStr">
         <is>
-          <t>BCiC data-entry / naming consistency; confirm identity of Financial Risk approver.</t>
+          <t>Mitigated by production vs test-day screenshots in BLA02, BCiC Y/Y/Y (E03) and signed attestation (DMA02 attachment).</t>
         </is>
       </c>
       <c r="F74" s="87" t="inlineStr"/>
@@ -7297,26 +7347,26 @@
     </row>
     <row r="75" ht="42" customHeight="1" s="71">
       <c r="A75" s="87" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B75" s="87" t="inlineStr">
         <is>
-          <t>ACH Express and Interface Monitor are not named verbatim in the DIV "Application In-scope" lines of BLA01 / BLA04; BLA01 operator (Raimy Ayala) differs from BCiC tester (Andreina De Stefano).</t>
+          <t>BSA T24 record (E03 row 8) Attestation Date 08/29/2026 vs signed attestation 8/19/2026 (DMA02 attachment); Financial Risk manager recorded as "Xavier Caisapanta" in BCiC while the approval email is from Ivan Caisapanta (DMA08).</t>
         </is>
       </c>
       <c r="C75" s="87" t="inlineStr">
         <is>
-          <t>1822, 4052, 1867, 1868</t>
+          <t>1937</t>
         </is>
       </c>
       <c r="D75" s="87" t="inlineStr">
         <is>
-          <t>BLA01, BLA04, E03, MA01</t>
+          <t>E03, DMA02, DMA08</t>
         </is>
       </c>
       <c r="E75" s="87" t="inlineStr">
         <is>
-          <t>Application-level DIV records exist in BCiC (E03 rows 47 and 61) with Y/Y/Y results and manager approval.</t>
+          <t>BCiC data-entry / naming consistency; confirm identity of Financial Risk approver.</t>
         </is>
       </c>
       <c r="F75" s="87" t="inlineStr"/>
@@ -7334,28 +7384,28 @@
       <c r="R75" s="82" t="n"/>
       <c r="S75" s="82" t="n"/>
     </row>
-    <row r="76" ht="54" customHeight="1" s="71">
+    <row r="76" ht="30" customHeight="1" s="71">
       <c r="A76" s="87" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B76" s="87" t="inlineStr">
         <is>
-          <t>Count reconciliation – E03 contains 62 DIV records (56 for the 10 tested applications); E16b contains 64 rows (one additional Treasury T24 row with blank department, row 45); the attestation states 63 entries / 13 applications.</t>
+          <t>ACH Express and Interface Monitor are not named verbatim in the DIV "Application In-scope" lines of BLA01 / BLA04; BLA01 operator (Raimy Ayala) differs from BCiC tester (Andreina De Stefano).</t>
         </is>
       </c>
       <c r="C76" s="87" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>1822, 4052, 1867, 1868</t>
         </is>
       </c>
       <c r="D76" s="87" t="inlineStr">
         <is>
-          <t>E03, E16b, DMA02</t>
+          <t>BLA01, BLA04, E03, MA01</t>
         </is>
       </c>
       <c r="E76" s="87" t="inlineStr">
         <is>
-          <t>Testing performed on E03 (the export containing the manager approval fields).</t>
+          <t>Application-level DIV records exist in BCiC (E03 rows 47 and 61) with Y/Y/Y results and manager approval.</t>
         </is>
       </c>
       <c r="F76" s="87" t="inlineStr"/>
@@ -7373,13 +7423,13 @@
       <c r="R76" s="82" t="n"/>
       <c r="S76" s="82" t="n"/>
     </row>
-    <row r="77" ht="30" customHeight="1" s="71">
+    <row r="77" ht="42" customHeight="1" s="71">
       <c r="A77" s="87" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B77" s="87" t="inlineStr">
         <is>
-          <t>Annual interval – prior DR exercise 10/19/2024 to 11/15/2025 = 392 days; one exercise per annual DR cycle (2024, 2025) and within the review period.</t>
+          <t>Count reconciliation – E03 contains 62 DIV records (56 for the 10 tested applications); E16b contains 64 rows (one additional Treasury T24 row with blank department, row 45); the attestation states 63 entries / 13 applications.</t>
         </is>
       </c>
       <c r="C77" s="87" t="inlineStr">
@@ -7389,12 +7439,12 @@
       </c>
       <c r="D77" s="87" t="inlineStr">
         <is>
-          <t>Tab 'DR 2024 Testing Results'; E01; E03</t>
+          <t>E03, E16b, DMA02</t>
         </is>
       </c>
       <c r="E77" s="87" t="inlineStr">
         <is>
-          <t>Annual requirement assessed per DR cycle.</t>
+          <t>Testing performed on E03 (the export containing the manager approval fields).</t>
         </is>
       </c>
       <c r="F77" s="87" t="inlineStr"/>
@@ -7412,28 +7462,28 @@
       <c r="R77" s="82" t="n"/>
       <c r="S77" s="82" t="n"/>
     </row>
-    <row r="78" ht="102" customHeight="1" s="71">
+    <row r="78" ht="30" customHeight="1" s="71">
       <c r="A78" s="87" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B78" s="87" t="inlineStr">
         <is>
-          <t>Redundant files removed: 13 duplicate evidence files (byte-identical copies or the same email saved twice: E11, E12, E14, E14a, E15, E15a, E16, E16a, E17, E17a, MA02, DMA05b, E06) and the extracted attachment copies (8 signed attestation PDFs, 26 E07/E08 report files) and E06 (same meeting invite as E05, re-sent) were removed; each item is retained once – signed attestations and report files are cited through the email that contains them (see Evidence Index – files removed). E13 (11/13/2024) is prior period – supplemental only. DMA13 (Cisco Call Manager) is out of scope.</t>
+          <t>Annual interval – prior DR exercise 10/19/2024 to 11/15/2025 = 392 days; one exercise per annual DR cycle (2024, 2025) and within the review period.</t>
         </is>
       </c>
       <c r="C78" s="87" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>All</t>
         </is>
       </c>
       <c r="D78" s="87" t="inlineStr">
         <is>
-          <t>Evidence Index tab</t>
+          <t>Tab 'DR 2024 Testing Results'; E01; E03</t>
         </is>
       </c>
       <c r="E78" s="87" t="inlineStr">
         <is>
-          <t>No impact – retained copy carries identical content.</t>
+          <t>Annual requirement assessed per DR cycle.</t>
         </is>
       </c>
       <c r="F78" s="87" t="inlineStr"/>
@@ -7451,13 +7501,31 @@
       <c r="R78" s="82" t="n"/>
       <c r="S78" s="82" t="n"/>
     </row>
-    <row r="79" s="71">
-      <c r="A79" s="82" t="n"/>
-      <c r="B79" s="82" t="n"/>
-      <c r="C79" s="82" t="n"/>
-      <c r="D79" s="82" t="n"/>
-      <c r="E79" s="82" t="n"/>
-      <c r="F79" s="82" t="n"/>
+    <row r="79" ht="78" customHeight="1" s="71">
+      <c r="A79" s="87" t="n">
+        <v>9</v>
+      </c>
+      <c r="B79" s="87" t="inlineStr">
+        <is>
+          <t>Redundant files removed: 12 duplicate evidence files (byte-identical copies or the same email saved twice: E11, E12, E14, E14a, E15, E15a, E16, E16a, E17, E17a, DMA05b, E06) and the extracted attachment copies (8 signed attestation PDFs, 26 E07/E08 report files) and E06 (same meeting invite as E05, re-sent) were removed; each item is retained once – signed attestations and report files are cited through the email that contains them (see Evidence Index – files removed). E13 (11/13/2024) is prior period – supplemental only. DMA13 (Cisco Call Manager) is out of scope.</t>
+        </is>
+      </c>
+      <c r="C79" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D79" s="87" t="inlineStr">
+        <is>
+          <t>Evidence Index tab</t>
+        </is>
+      </c>
+      <c r="E79" s="87" t="inlineStr">
+        <is>
+          <t>No impact – retained copy carries identical content.</t>
+        </is>
+      </c>
+      <c r="F79" s="87" t="inlineStr"/>
       <c r="G79" s="82" t="n"/>
       <c r="H79" s="82" t="n"/>
       <c r="I79" s="82" t="n"/>
@@ -7472,12 +7540,19 @@
       <c r="R79" s="82" t="n"/>
       <c r="S79" s="82" t="n"/>
     </row>
-    <row r="80" ht="22" customHeight="1" s="71">
-      <c r="A80" s="73" t="inlineStr">
-        <is>
-          <t>Reviewer Note</t>
-        </is>
-      </c>
+    <row r="80" s="71">
+      <c r="A80" s="82" t="n"/>
+      <c r="B80" s="82" t="n"/>
+      <c r="C80" s="82" t="n"/>
+      <c r="D80" s="82" t="n"/>
+      <c r="E80" s="82" t="n"/>
+      <c r="F80" s="82" t="n"/>
+      <c r="G80" s="82" t="n"/>
+      <c r="H80" s="82" t="n"/>
+      <c r="I80" s="82" t="n"/>
+      <c r="J80" s="82" t="n"/>
+      <c r="K80" s="82" t="n"/>
+      <c r="L80" s="82" t="n"/>
       <c r="M80" s="82" t="n"/>
       <c r="N80" s="82" t="n"/>
       <c r="O80" s="82" t="n"/>
@@ -7486,10 +7561,10 @@
       <c r="R80" s="82" t="n"/>
       <c r="S80" s="82" t="n"/>
     </row>
-    <row r="81" ht="75" customHeight="1" s="71">
-      <c r="A81" s="88" t="inlineStr">
-        <is>
-          <t>All requested attributes (IT DR exercise name, annual execution, application, tester, business data validation, manager name/approval dates, DIV procedures, approval emails, BCiC evidence, Annual Testing Executed, DIV Performed by IT DR Team, Applications in Scope Identified, Business Line Approval of Results, Results Documented in BCMS, overall assessment, supporting evidence and sample result) are completed for the 10 in-scope applications (56 DIV records) and every conclusion is linked to its evidence file and folder location in BSI.IT.6.C7.3-Evidences. Applications in Scope Identified is based on MA01 (BSI In-Scope Applications-2026). Business Line Approval of Results is based on the Business Line Approval Results – Email folder (BLA01–BLA06) together with the application-specific approval emails / signed attestations (folder 03, E09).</t>
+    <row r="81" ht="22" customHeight="1" s="71">
+      <c r="A81" s="73" t="inlineStr">
+        <is>
+          <t>Reviewer Note</t>
         </is>
       </c>
       <c r="M81" s="82" t="n"/>
@@ -7500,19 +7575,12 @@
       <c r="R81" s="82" t="n"/>
       <c r="S81" s="82" t="n"/>
     </row>
-    <row r="82" s="71">
-      <c r="A82" s="82" t="n"/>
-      <c r="B82" s="82" t="n"/>
-      <c r="C82" s="82" t="n"/>
-      <c r="D82" s="82" t="n"/>
-      <c r="E82" s="82" t="n"/>
-      <c r="F82" s="82" t="n"/>
-      <c r="G82" s="82" t="n"/>
-      <c r="H82" s="82" t="n"/>
-      <c r="I82" s="82" t="n"/>
-      <c r="J82" s="82" t="n"/>
-      <c r="K82" s="82" t="n"/>
-      <c r="L82" s="82" t="n"/>
+    <row r="82" ht="75" customHeight="1" s="71">
+      <c r="A82" s="88" t="inlineStr">
+        <is>
+          <t>All requested attributes (IT DR exercise name, annual execution, application, tester, business data validation, manager name/approval dates, DIV procedures, approval emails, BCiC evidence, Annual Testing Executed, DIV Performed by IT DR Team, Applications in Scope Identified, Business Line Approval of Results, Results Documented in BCMS, overall assessment, supporting evidence and sample result) are completed for the 10 in-scope applications (56 DIV records) and every conclusion is linked to its evidence file and folder location in BSI.IT.6.C7.3-Evidences. Applications in Scope Identified is based on MA01 (BSI In-Scope Applications-2026). Business Line Approval of Results is based on the Business Line Approval Results – Email folder (BLA01–BLA06) together with the application-specific approval emails / signed attestations (folder 03, E09).</t>
+        </is>
+      </c>
       <c r="M82" s="82" t="n"/>
       <c r="N82" s="82" t="n"/>
       <c r="O82" s="82" t="n"/>
@@ -8743,12 +8811,12 @@
   <mergeCells count="8">
     <mergeCell ref="A81:L81"/>
     <mergeCell ref="A15:L15"/>
-    <mergeCell ref="A68:L68"/>
+    <mergeCell ref="A82:L82"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A28:L28"/>
     <mergeCell ref="A37:L37"/>
-    <mergeCell ref="A80:L80"/>
     <mergeCell ref="A53:L53"/>
+    <mergeCell ref="A69:L69"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
@@ -8990,6 +9058,7 @@
       <c r="M5" s="62" t="inlineStr">
         <is>
           <t>• MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png – BSI In-Scope Applications-2026 – App ID 1822 selected; 2025 DR Test Scope, 2025 Backup/Restore Test Scope and 2025 Backup/Restore DIV Scope = True
+• MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg – Management Attestation email 08/18/2026 – attached signed attestation (4069_001.pdf) §2 lists the 13 in-scope applications that store business data, including this application
 • E01 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx – row 3 – 2025 DR Test Scope = True; 2025 Backup/Restore DIV Scope = True
 • E02 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg – view 'Applications In Scope for DR Test BSI'
 • E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg – BIA results &amp; applications list review
@@ -9015,8 +9084,9 @@
       </c>
       <c r="P5" s="62" t="inlineStr">
         <is>
-          <t>[01 Management Attestation / In-Scope Applications]
+          <t xml:space="preserve">[01 Management Attestation / In-Scope Applications]
 MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png
+MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg
 [02 Business Line Approval Results – Email]
 BLA01 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf
 [03 DIV Manager Attestation Email Approvals]
@@ -9029,12 +9099,13 @@
 E04 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg
 E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg
 E09 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg
-E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx
+</t>
         </is>
       </c>
       <c r="Q5" s="62" t="inlineStr">
         <is>
-          <t>PASS – with observations – MA01, BLA01, DMA01, DMA02, E01, E02, E03, E04, E05, E09, E16b</t>
+          <t>PASS – with observations – MA01, MA02, BLA01, DMA01, DMA02, E01, E02, E03, E04, E05, E09, E16b</t>
         </is>
       </c>
     </row>
@@ -9137,6 +9208,7 @@
       <c r="M6" s="62" t="inlineStr">
         <is>
           <t>• MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png – BSI In-Scope Applications-2026 – App ID 1867 selected; 2025 DR Test Scope, 2025 Backup/Restore Test Scope and 2025 Backup/Restore DIV Scope = True
+• MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg – Management Attestation email 08/18/2026 – attached signed attestation (4069_001.pdf) §2 lists the 13 in-scope applications that store business data, including this application
 • E01 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx – row 19 – 2025 DR Test Scope = True; 2025 Backup/Restore DIV Scope = True
 • E02 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg – view 'Applications In Scope for DR Test BSI'
 • E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg – BIA results &amp; applications list review
@@ -9162,8 +9234,9 @@
       </c>
       <c r="P6" s="62" t="inlineStr">
         <is>
-          <t>[01 Management Attestation / In-Scope Applications]
+          <t xml:space="preserve">[01 Management Attestation / In-Scope Applications]
 MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png
+MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg
 [02 Business Line Approval Results – Email]
 BLA01 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf
 [03 DIV Manager Attestation Email Approvals]
@@ -9176,12 +9249,13 @@
 E04 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg
 E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg
 E09 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg
-E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx
+</t>
         </is>
       </c>
       <c r="Q6" s="62" t="inlineStr">
         <is>
-          <t>PASS – with observations – MA01, BLA01, DMA01, DMA02, E01, E02, E03, E04, E05, E09, E16b</t>
+          <t>PASS – with observations – MA01, MA02, BLA01, DMA01, DMA02, E01, E02, E03, E04, E05, E09, E16b</t>
         </is>
       </c>
     </row>
@@ -9284,6 +9358,7 @@
       <c r="M7" s="62" t="inlineStr">
         <is>
           <t>• MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png – BSI In-Scope Applications-2026 – App ID 1868 selected; 2025 DR Test Scope, 2025 Backup/Restore Test Scope and 2025 Backup/Restore DIV Scope = True
+• MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg – Management Attestation email 08/18/2026 – attached signed attestation (4069_001.pdf) §2 lists the 13 in-scope applications that store business data, including this application
 • E01 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx – row 20 – 2025 DR Test Scope = True; 2025 Backup/Restore DIV Scope = True
 • E02 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg – view 'Applications In Scope for DR Test BSI'
 • E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg – BIA results &amp; applications list review
@@ -9309,8 +9384,9 @@
       </c>
       <c r="P7" s="62" t="inlineStr">
         <is>
-          <t>[01 Management Attestation / In-Scope Applications]
+          <t xml:space="preserve">[01 Management Attestation / In-Scope Applications]
 MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png
+MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg
 [02 Business Line Approval Results – Email]
 BLA01 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf
 [03 DIV Manager Attestation Email Approvals]
@@ -9323,12 +9399,13 @@
 E04 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg
 E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg
 E09 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg
-E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx
+</t>
         </is>
       </c>
       <c r="Q7" s="62" t="inlineStr">
         <is>
-          <t>PASS – with observations – MA01, BLA01, DMA01, DMA02, E01, E02, E03, E04, E05, E09, E16b</t>
+          <t>PASS – with observations – MA01, MA02, BLA01, DMA01, DMA02, E01, E02, E03, E04, E05, E09, E16b</t>
         </is>
       </c>
     </row>
@@ -9446,6 +9523,7 @@
       <c r="M8" s="62" t="inlineStr">
         <is>
           <t>• MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png – BSI In-Scope Applications-2026 – App ID 3299 selected; 2025 DR Test Scope, 2025 Backup/Restore Test Scope and 2025 Backup/Restore DIV Scope = True
+• MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg – Management Attestation email 08/18/2026 – attached signed attestation (4069_001.pdf) §2 lists the 13 in-scope applications that store business data, including this application
 • E01 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx – row 24 – 2025 DR Test Scope = True; 2025 Backup/Restore DIV Scope = True
 • E02 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg – view 'Applications In Scope for DR Test BSI'
 • E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg – BIA results &amp; applications list review
@@ -9475,8 +9553,9 @@
       </c>
       <c r="P8" s="62" t="inlineStr">
         <is>
-          <t>[01 Management Attestation / In-Scope Applications]
+          <t xml:space="preserve">[01 Management Attestation / In-Scope Applications]
 MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png
+MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg
 [02 Business Line Approval Results – Email]
 BLA01 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf
 BLA02 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf
@@ -9492,12 +9571,13 @@
 E04 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg
 E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg
 E09 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg
-E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx
+</t>
         </is>
       </c>
       <c r="Q8" s="62" t="inlineStr">
         <is>
-          <t>PASS – with observations – MA01, BLA01, BLA02, DMA01, DMA02, DMA05, DMA11, E01, E02, E03, E04, E05, E09, E16b</t>
+          <t>PASS – with observations – MA01, MA02, BLA01, BLA02, DMA01, DMA02, DMA05, DMA11, E01, E02, E03, E04, E05, E09, E16b</t>
         </is>
       </c>
     </row>
@@ -9591,6 +9671,7 @@
       <c r="M9" s="62" t="inlineStr">
         <is>
           <t>• MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png – BSI In-Scope Applications-2026 – App ID 4052 selected; 2025 DR Test Scope, 2025 Backup/Restore Test Scope and 2025 Backup/Restore DIV Scope = True
+• MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg – Management Attestation email 08/18/2026 – attached signed attestation (4069_001.pdf) §2 lists the 13 in-scope applications that store business data, including this application
 • E01 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx – row 25 – 2025 DR Test Scope = True; 2025 Backup/Restore DIV Scope = True
 • E02 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg – view 'Applications In Scope for DR Test BSI'
 • E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg – BIA results &amp; applications list review
@@ -9614,8 +9695,9 @@
       </c>
       <c r="P9" s="62" t="inlineStr">
         <is>
-          <t>[01 Management Attestation / In-Scope Applications]
+          <t xml:space="preserve">[01 Management Attestation / In-Scope Applications]
 MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png
+MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg
 [02 Business Line Approval Results – Email]
 BLA04 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx
 [03 DIV Manager Attestation Email Approvals]
@@ -9627,12 +9709,13 @@
 E03 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls
 E04 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg
 E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg
-E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx
+</t>
         </is>
       </c>
       <c r="Q9" s="62" t="inlineStr">
         <is>
-          <t>PASS – with observations – MA01, BLA04, DMA02, DMA04, E01, E02, E03, E04, E05, E16b</t>
+          <t>PASS – with observations – MA01, MA02, BLA04, DMA02, DMA04, E01, E02, E03, E04, E05, E16b</t>
         </is>
       </c>
     </row>
@@ -9729,6 +9812,7 @@
       <c r="M10" s="62" t="inlineStr">
         <is>
           <t>• MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png – BSI In-Scope Applications-2026 – App ID 3301 selected; 2025 DR Test Scope, 2025 Backup/Restore Test Scope and 2025 Backup/Restore DIV Scope = True
+• MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg – Management Attestation email 08/18/2026 – attached signed attestation (4069_001.pdf) §2 lists the 13 in-scope applications that store business data, including this application
 • E01 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx – row 31 – 2025 DR Test Scope = True; 2025 Backup/Restore DIV Scope = True
 • E02 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg – view 'Applications In Scope for DR Test BSI'
 • E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg – BIA results &amp; applications list review
@@ -9752,8 +9836,9 @@
       </c>
       <c r="P10" s="62" t="inlineStr">
         <is>
-          <t>[01 Management Attestation / In-Scope Applications]
+          <t xml:space="preserve">[01 Management Attestation / In-Scope Applications]
 MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png
+MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg
 [02 Business Line Approval Results – Email]
 BLA03 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf
 [03 DIV Manager Attestation Email Approvals]
@@ -9767,12 +9852,13 @@
 E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg
 E07 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg
 E08 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg
-E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx
+</t>
         </is>
       </c>
       <c r="Q10" s="62" t="inlineStr">
         <is>
-          <t>PASS – with observations – MA01, BLA03, DMA02, DMA03, E01, E02, E03, E04, E05, E07, E08, E16b</t>
+          <t>PASS – with observations – MA01, MA02, BLA03, DMA02, DMA03, E01, E02, E03, E04, E05, E07, E08, E16b</t>
         </is>
       </c>
     </row>
@@ -9885,6 +9971,7 @@
       <c r="M11" s="62" t="inlineStr">
         <is>
           <t>• MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png – BSI In-Scope Applications-2026 – App ID 1903 selected; 2025 DR Test Scope, 2025 Backup/Restore Test Scope and 2025 Backup/Restore DIV Scope = True
+• MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg – Management Attestation email 08/18/2026 – attached signed attestation (4069_001.pdf) §2 lists the 13 in-scope applications that store business data, including this application
 • E01 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx – row 34 – 2025 DR Test Scope = True; 2025 Backup/Restore DIV Scope = True
 • E02 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg – view 'Applications In Scope for DR Test BSI'
 • E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg – BIA results &amp; applications list review
@@ -9911,8 +9998,9 @@
       </c>
       <c r="P11" s="62" t="inlineStr">
         <is>
-          <t>[01 Management Attestation / In-Scope Applications]
+          <t xml:space="preserve">[01 Management Attestation / In-Scope Applications]
 MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png
+MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg
 [02 Business Line Approval Results – Email]
 BLA02 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf
 BLA03 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf
@@ -9928,12 +10016,13 @@
 E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg
 E07 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg
 E08 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg
-E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx
+</t>
         </is>
       </c>
       <c r="Q11" s="62" t="inlineStr">
         <is>
-          <t>PASS – with observations – MA01, BLA02, BLA03, DMA02, DMA03, DMA05, E01, E02, E03, E04, E05, E07, E08, E16b</t>
+          <t>PASS – with observations – MA01, MA02, BLA02, BLA03, DMA02, DMA03, DMA05, E01, E02, E03, E04, E05, E07, E08, E16b</t>
         </is>
       </c>
     </row>
@@ -10028,6 +10117,7 @@
       <c r="M12" s="62" t="inlineStr">
         <is>
           <t>• MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png – BSI In-Scope Applications-2026 – App ID 1917 selected; 2025 DR Test Scope, 2025 Backup/Restore Test Scope and 2025 Backup/Restore DIV Scope = True
+• MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg – Management Attestation email 08/18/2026 – attached signed attestation (4069_001.pdf) §2 lists the 13 in-scope applications that store business data, including this application
 • E01 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx – row 36 – 2025 DR Test Scope = True; 2025 Backup/Restore DIV Scope = True
 • E02 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg – view 'Applications In Scope for DR Test BSI'
 • E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg – BIA results &amp; applications list review
@@ -10051,8 +10141,9 @@
       </c>
       <c r="P12" s="62" t="inlineStr">
         <is>
-          <t>[01 Management Attestation / In-Scope Applications]
+          <t xml:space="preserve">[01 Management Attestation / In-Scope Applications]
 MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png
+MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg
 [02 Business Line Approval Results – Email]
 BLA05 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf
 BLA06 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg
@@ -10065,12 +10156,13 @@
 E04 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg
 E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg
 E10 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg
-E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx
+</t>
         </is>
       </c>
       <c r="Q12" s="62" t="inlineStr">
         <is>
-          <t>PASS – with observations – MA01, BLA05, BLA06, DMA02, E01, E02, E03, E04, E05, E10, E16b</t>
+          <t>PASS – with observations – MA01, MA02, BLA05, BLA06, DMA02, E01, E02, E03, E04, E05, E10, E16b</t>
         </is>
       </c>
     </row>
@@ -10180,6 +10272,7 @@
       <c r="M13" s="62" t="inlineStr">
         <is>
           <t>• MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png – BSI In-Scope Applications-2026 – App ID 1936 selected; 2025 DR Test Scope, 2025 Backup/Restore Test Scope and 2025 Backup/Restore DIV Scope = True
+• MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg – Management Attestation email 08/18/2026 – attached signed attestation (4069_001.pdf) §2 lists the 13 in-scope applications that store business data, including this application
 • E01 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx – row 42 – 2025 DR Test Scope = True; 2025 Backup/Restore DIV Scope = True
 • E02 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg – view 'Applications In Scope for DR Test BSI'
 • E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg – BIA results &amp; applications list review
@@ -10205,8 +10298,9 @@
       </c>
       <c r="P13" s="62" t="inlineStr">
         <is>
-          <t>[01 Management Attestation / In-Scope Applications]
+          <t xml:space="preserve">[01 Management Attestation / In-Scope Applications]
 MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png
+MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg
 [02 Business Line Approval Results – Email]
 BLA03 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf
 BLA04 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx
@@ -10221,12 +10315,13 @@
 E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg
 E07 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg
 E08 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg
-E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx
+</t>
         </is>
       </c>
       <c r="Q13" s="62" t="inlineStr">
         <is>
-          <t>PASS – with observations – MA01, BLA03, BLA04, DMA02, DMA04, E01, E02, E03, E04, E05, E07, E08, E16b</t>
+          <t>PASS – with observations – MA01, MA02, BLA03, BLA04, DMA02, DMA04, E01, E02, E03, E04, E05, E07, E08, E16b</t>
         </is>
       </c>
     </row>
@@ -10391,6 +10486,7 @@
       <c r="M14" s="62" t="inlineStr">
         <is>
           <t>• MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png – BSI In-Scope Applications-2026 – App ID 1937 selected; 2025 DR Test Scope, 2025 Backup/Restore Test Scope and 2025 Backup/Restore DIV Scope = True
+• MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg – Management Attestation email 08/18/2026 – attached signed attestation (4069_001.pdf) §2 lists the 13 in-scope applications that store business data, including this application
 • E01 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx – row 43 – 2025 DR Test Scope = True; 2025 Backup/Restore DIV Scope = True
 • E02 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg – view 'Applications In Scope for DR Test BSI'
 • E05 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg – BIA results &amp; applications list review
@@ -10431,8 +10527,9 @@
       </c>
       <c r="P14" s="62" t="inlineStr">
         <is>
-          <t>[01 Management Attestation / In-Scope Applications]
+          <t xml:space="preserve">[01 Management Attestation / In-Scope Applications]
 MA01 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA01_BSI In-Scope Applications-2026.png
+MA02 – BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg
 [02 Business Line Approval Results – Email]
 BLA01 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf
 BLA02 – BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email\BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf
@@ -10463,12 +10560,13 @@
 E08 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg
 E09 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg
 E10 – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg
-E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+E16b – BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence\BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx
+</t>
         </is>
       </c>
       <c r="Q14" s="62" t="inlineStr">
         <is>
-          <t>PASS – with observations – MA01, BLA01, BLA02, BLA03, BLA04, BLA05, BLA06, DMA01, DMA02, DMA03, DMA04, DMA05, DMA06, DMA07, DMA08, DMA09, DMA10, DMA11, DMA12, E01, E02, E03, E04, E05, E07, E08, E09, E10, E16b</t>
+          <t>PASS – with observations – MA01, MA02, BLA01, BLA02, BLA03, BLA04, BLA05, BLA06, DMA01, DMA02, DMA03, DMA04, DMA05, DMA06, DMA07, DMA08, DMA09, DMA10, DMA11, DMA12, E01, E02, E03, E04, E05, E07, E08, E09, E10, E16b</t>
         </is>
       </c>
     </row>
@@ -13007,52 +13105,52 @@
     <row r="4" ht="34.5" customHeight="1" s="71">
       <c r="A4" s="64" t="inlineStr">
         <is>
-          <t>BLA01</t>
+          <t>MA02</t>
         </is>
       </c>
       <c r="B4" s="64" t="inlineStr">
         <is>
-          <t>BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf</t>
+          <t>MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg</t>
         </is>
       </c>
       <c r="C4" s="64" t="inlineStr">
         <is>
-          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email</t>
+          <t>BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications</t>
         </is>
       </c>
       <c r="D4" s="64" t="inlineStr">
         <is>
-          <t>Client Back Office - FED inclearing ACH  Cash letter (1).pdf</t>
+          <t>RE_ Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises) 3 (2).msg</t>
         </is>
       </c>
       <c r="E4" s="64" t="inlineStr">
         <is>
-          <t>Business Line Approval Results - Email.zip</t>
+          <t>Management_Attestation.zip</t>
         </is>
       </c>
       <c r="F4" s="64" t="inlineStr">
         <is>
-          <t>DR test script / DIV test results</t>
+          <t>Email + signed management attestation</t>
         </is>
       </c>
       <c r="G4" s="64" t="inlineStr">
         <is>
-          <t>11/15/2025 – Client Back Office (operator Raimy Ayala)</t>
+          <t>08/18/2026 – Frank Puentes</t>
         </is>
       </c>
       <c r="H4" s="64" t="inlineStr">
         <is>
-          <t>DR test script with Data Integrity Validation section. Application in-scope: FedImport, FedExport, Imaging101, T24. Format / Headers / Content = Y – "No data discrepancy found". Steps include ACH Express import and Imaging101 validation screenshots (14 pages).</t>
+          <t>Management Attestation email: Frank Puentes (Executive Director, Payments &amp; Cash Management) returns the signed attestation (attachment 4069_001.pdf) to Cesar Vidal. The quoted Cesar Vidal request (08/17/2026) confirms the DR exercises of 11/15/2025 and 02/21/2026 and attaches the BCiC DIV export; the signed attestation §2 lists the 13 in-scope BSI applications that store business data, including all 10 tested applications. Filed in the Management_Attestation folder as received; the same message is also filed as DMA03 for the business line approval attribute.</t>
         </is>
       </c>
       <c r="I4" s="64" t="inlineStr">
         <is>
-          <t>1822, 1867, 1868, 3299, 1937</t>
+          <t>1822, 1867, 1868, 3299, 4052, 3301, 1903, 1917, 1936, 1937</t>
         </is>
       </c>
       <c r="J4" s="64" t="inlineStr">
         <is>
-          <t>B, E, F, I, L, M, O</t>
+          <t>N</t>
         </is>
       </c>
       <c r="K4" s="64" t="inlineStr"/>
@@ -13061,12 +13159,12 @@
     <row r="5" ht="34.5" customHeight="1" s="71">
       <c r="A5" s="64" t="inlineStr">
         <is>
-          <t>BLA02</t>
+          <t>BLA01</t>
         </is>
       </c>
       <c r="B5" s="64" t="inlineStr">
         <is>
-          <t>BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf</t>
+          <t>BLA01_Client Back Office - FED Inclearing ACH &amp; Cash Letter - DIV Test Results 11-15-2025.pdf</t>
         </is>
       </c>
       <c r="C5" s="64" t="inlineStr">
@@ -13076,7 +13174,7 @@
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
-          <t>BSA_AML_OFAC Compliance - DM 11.15.2025 (002) (1).pdf</t>
+          <t>Client Back Office - FED inclearing ACH  Cash letter (1).pdf</t>
         </is>
       </c>
       <c r="E5" s="64" t="inlineStr">
@@ -13091,17 +13189,17 @@
       </c>
       <c r="G5" s="64" t="inlineStr">
         <is>
-          <t>11/15/2025 – BSA/AML/OFAC Compliance (operator David Marquez)</t>
+          <t>11/15/2025 – Client Back Office (operator Raimy Ayala)</t>
         </is>
       </c>
       <c r="H5" s="64" t="inlineStr">
         <is>
-          <t>OFAC Verifier test script. Application in-scope: T24, Imaging101, OFAC. DIV procedure instructions listed; production-day (11/14/2025) vs test-day (11/15/2025) screenshots for T24, Imaging101/ModeloIC and OFAC Report 64. NOTE: DIV Yes/No answer boxes on p.1 are blank.</t>
+          <t>DR test script with Data Integrity Validation section. Application in-scope: FedImport, FedExport, Imaging101, T24. Format / Headers / Content = Y – "No data discrepancy found". Steps include ACH Express import and Imaging101 validation screenshots (14 pages).</t>
         </is>
       </c>
       <c r="I5" s="64" t="inlineStr">
         <is>
-          <t>3299, 1903, 1937</t>
+          <t>1822, 1867, 1868, 3299, 1937</t>
         </is>
       </c>
       <c r="J5" s="64" t="inlineStr">
@@ -13115,12 +13213,12 @@
     <row r="6" ht="69" customHeight="1" s="71">
       <c r="A6" s="64" t="inlineStr">
         <is>
-          <t>BLA03</t>
+          <t>BLA02</t>
         </is>
       </c>
       <c r="B6" s="64" t="inlineStr">
         <is>
-          <t>BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf</t>
+          <t>BLA02_BSA_AML_OFAC Compliance - OFAC Verifier - DIV Test Results 11-15-2025.pdf</t>
         </is>
       </c>
       <c r="C6" s="64" t="inlineStr">
@@ -13130,7 +13228,7 @@
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>PAYMENTS SCRIPT NOV 2025.pdf</t>
+          <t>BSA_AML_OFAC Compliance - DM 11.15.2025 (002) (1).pdf</t>
         </is>
       </c>
       <c r="E6" s="64" t="inlineStr">
@@ -13145,17 +13243,17 @@
       </c>
       <c r="G6" s="64" t="inlineStr">
         <is>
-          <t>11/15/2025 – Payments &amp; Position Management (operators Frank Puentes / Gustavo Bucaro)</t>
+          <t>11/15/2025 – BSA/AML/OFAC Compliance (operator David Marquez)</t>
         </is>
       </c>
       <c r="H6" s="64" t="inlineStr">
         <is>
-          <t>Wire Transfer / Cash Mgt / Financial Messaging script. DIV application in-scope: T24, MQ Payment Monitor, OFAC – BSI, Fedlink – BSI, Swift Interface – BSI. Format / Headers / Content = yes; data from 11/14/2025 Fed &amp; SWIFT reconciled.</t>
+          <t>OFAC Verifier test script. Application in-scope: T24, Imaging101, OFAC. DIV procedure instructions listed; production-day (11/14/2025) vs test-day (11/15/2025) screenshots for T24, Imaging101/ModeloIC and OFAC Report 64. NOTE: DIV Yes/No answer boxes on p.1 are blank.</t>
         </is>
       </c>
       <c r="I6" s="64" t="inlineStr">
         <is>
-          <t>3301, 1903, 1936, 1937</t>
+          <t>3299, 1903, 1937</t>
         </is>
       </c>
       <c r="J6" s="64" t="inlineStr">
@@ -13169,12 +13267,12 @@
     <row r="7" ht="46" customHeight="1" s="71">
       <c r="A7" s="64" t="inlineStr">
         <is>
-          <t>BLA04</t>
+          <t>BLA03</t>
         </is>
       </c>
       <c r="B7" s="64" t="inlineStr">
         <is>
-          <t>BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx</t>
+          <t>BLA03_Payments &amp; Cash Management - Payments Script - DIV Test Results 11-15-2025.pdf</t>
         </is>
       </c>
       <c r="C7" s="64" t="inlineStr">
@@ -13184,7 +13282,7 @@
       </c>
       <c r="D7" s="64" t="inlineStr">
         <is>
-          <t>Investment Operations- Treasury Hub &amp; Derivatives Operations (1).docx</t>
+          <t>PAYMENTS SCRIPT NOV 2025.pdf</t>
         </is>
       </c>
       <c r="E7" s="64" t="inlineStr">
@@ -13199,17 +13297,17 @@
       </c>
       <c r="G7" s="64" t="inlineStr">
         <is>
-          <t>11/15/2025 – Investment Operations (operator Michelle Oropesa)</t>
+          <t>11/15/2025 – Payments &amp; Position Management (operators Frank Puentes / Gustavo Bucaro)</t>
         </is>
       </c>
       <c r="H7" s="64" t="inlineStr">
         <is>
-          <t>Treasury Hub &amp; Derivatives Operations script. Systems accessed: Swift Interface Monitor – BSI, T24, MS Office, DTCC. DIV application in-scope: T24 &amp; Swift Interface – BSI. Incoming MT300 and FX S reports matched 11/14 vs 11/15; Format / Headers / Content = Yes.</t>
+          <t>Wire Transfer / Cash Mgt / Financial Messaging script. DIV application in-scope: T24, MQ Payment Monitor, OFAC – BSI, Fedlink – BSI, Swift Interface – BSI. Format / Headers / Content = yes; data from 11/14/2025 Fed &amp; SWIFT reconciled.</t>
         </is>
       </c>
       <c r="I7" s="64" t="inlineStr">
         <is>
-          <t>4052, 1936, 1937</t>
+          <t>3301, 1903, 1936, 1937</t>
         </is>
       </c>
       <c r="J7" s="64" t="inlineStr">
@@ -13223,12 +13321,12 @@
     <row r="8" ht="23" customHeight="1" s="71">
       <c r="A8" s="64" t="inlineStr">
         <is>
-          <t>BLA05</t>
+          <t>BLA04</t>
         </is>
       </c>
       <c r="B8" s="64" t="inlineStr">
         <is>
-          <t>BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf</t>
+          <t>BLA04_Investment Operations - Treasury Hub &amp; Derivatives Operations - DIV Test Results 11-15-2025.docx</t>
         </is>
       </c>
       <c r="C8" s="64" t="inlineStr">
@@ -13238,7 +13336,7 @@
       </c>
       <c r="D8" s="64" t="inlineStr">
         <is>
-          <t>Financial Analysis and Control-GL (1).pdf</t>
+          <t>Investment Operations- Treasury Hub &amp; Derivatives Operations (1).docx</t>
         </is>
       </c>
       <c r="E8" s="64" t="inlineStr">
@@ -13253,17 +13351,17 @@
       </c>
       <c r="G8" s="64" t="inlineStr">
         <is>
-          <t>11/15/2025 – Finance &amp; Accounting Reporting (operator Dunia Gonzalez Collado)</t>
+          <t>11/15/2025 – Investment Operations (operator Michelle Oropesa)</t>
         </is>
       </c>
       <c r="H8" s="64" t="inlineStr">
         <is>
-          <t>General ledger review script. DIV application in-scope: T24 &amp; ReconXpert. Reconciliations passed; Format / Headers / Content = Yes, "No discrepancies found on the report".</t>
+          <t>Treasury Hub &amp; Derivatives Operations script. Systems accessed: Swift Interface Monitor – BSI, T24, MS Office, DTCC. DIV application in-scope: T24 &amp; Swift Interface – BSI. Incoming MT300 and FX S reports matched 11/14 vs 11/15; Format / Headers / Content = Yes.</t>
         </is>
       </c>
       <c r="I8" s="64" t="inlineStr">
         <is>
-          <t>1917, 1937</t>
+          <t>4052, 1936, 1937</t>
         </is>
       </c>
       <c r="J8" s="64" t="inlineStr">
@@ -13277,12 +13375,12 @@
     <row r="9" ht="23" customHeight="1" s="71">
       <c r="A9" s="64" t="inlineStr">
         <is>
-          <t>BLA06</t>
+          <t>BLA05</t>
         </is>
       </c>
       <c r="B9" s="64" t="inlineStr">
         <is>
-          <t>BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg</t>
+          <t>BLA05_Financial Analysis and Control - GL ReconXpert - DIV Test Results 11-15-2025.pdf</t>
         </is>
       </c>
       <c r="C9" s="64" t="inlineStr">
@@ -13292,7 +13390,7 @@
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>RE_ Testing enviroment.msg</t>
+          <t>Financial Analysis and Control-GL (1).pdf</t>
         </is>
       </c>
       <c r="E9" s="64" t="inlineStr">
@@ -13302,17 +13400,17 @@
       </c>
       <c r="F9" s="64" t="inlineStr">
         <is>
-          <t>Email approval</t>
+          <t>DR test script / DIV test results</t>
         </is>
       </c>
       <c r="G9" s="64" t="inlineStr">
         <is>
-          <t>12/31/2025 &amp; 01/26/2026 – Sadis Alvarenga</t>
+          <t>11/15/2025 – Finance &amp; Accounting Reporting (operator Dunia Gonzalez Collado)</t>
         </is>
       </c>
       <c r="H9" s="64" t="inlineStr">
         <is>
-          <t>Sadis Alvarenga (Financial Analysis &amp; Control manager) replies "Approved." on 12/31/2025 and again on 01/26/2026 to Elizabeth Noda's request to approve the submitted test script.</t>
+          <t>General ledger review script. DIV application in-scope: T24 &amp; ReconXpert. Reconciliations passed; Format / Headers / Content = Yes, "No discrepancies found on the report".</t>
         </is>
       </c>
       <c r="I9" s="64" t="inlineStr">
@@ -13322,7 +13420,7 @@
       </c>
       <c r="J9" s="64" t="inlineStr">
         <is>
-          <t>G, H, J, O</t>
+          <t>B, E, F, I, L, M, O</t>
         </is>
       </c>
       <c r="K9" s="64" t="inlineStr"/>
@@ -13331,47 +13429,47 @@
     <row r="10" ht="34.5" customHeight="1" s="71">
       <c r="A10" s="64" t="inlineStr">
         <is>
-          <t>DMA01</t>
+          <t>BLA06</t>
         </is>
       </c>
       <c r="B10" s="64" t="inlineStr">
         <is>
-          <t>DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg</t>
+          <t>BLA06_RE_ Testing enviroment - Financial Analysis Manager Approval - Sadis Alvarenga 01-26-2026.msg</t>
         </is>
       </c>
       <c r="C10" s="64" t="inlineStr">
         <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
+          <t>BSI.IT.6.C7.3-Evidences\02_Business_Line_Approval_Results_Email</t>
         </is>
       </c>
       <c r="D10" s="64" t="inlineStr">
         <is>
-          <t>RE_ Management Attestation – DIV Client Back Office.msg</t>
+          <t>RE_ Testing enviroment.msg</t>
         </is>
       </c>
       <c r="E10" s="64" t="inlineStr">
         <is>
-          <t>DIV Manager Attestation Email_Approvals.zip</t>
+          <t>Business Line Approval Results - Email.zip</t>
         </is>
       </c>
       <c r="F10" s="64" t="inlineStr">
         <is>
-          <t>Email attestation</t>
+          <t>Email approval</t>
         </is>
       </c>
       <c r="G10" s="64" t="inlineStr">
         <is>
-          <t>08/18/2026 – Claudia Romero</t>
+          <t>12/31/2025 &amp; 01/26/2026 – Sadis Alvarenga</t>
         </is>
       </c>
       <c r="H10" s="64" t="inlineStr">
         <is>
-          <t>Claudia Romero (Client Back Office Manager VP) returns the signed Management Attestation – attachment: Data_Integrity_Attestation_Santander-BCiC (002).pdf (signed Claudia Romero).</t>
+          <t>Sadis Alvarenga (Financial Analysis &amp; Control manager) replies "Approved." on 12/31/2025 and again on 01/26/2026 to Elizabeth Noda's request to approve the submitted test script.</t>
         </is>
       </c>
       <c r="I10" s="64" t="inlineStr">
         <is>
-          <t>1822, 1867, 1868, 3299, 1937</t>
+          <t>1917, 1937</t>
         </is>
       </c>
       <c r="J10" s="64" t="inlineStr">
@@ -13385,12 +13483,12 @@
     <row r="11" ht="23" customHeight="1" s="71">
       <c r="A11" s="64" t="inlineStr">
         <is>
-          <t>DMA02</t>
+          <t>DMA01</t>
         </is>
       </c>
       <c r="B11" s="64" t="inlineStr">
         <is>
-          <t>DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg</t>
+          <t>DMA01_RE_ Management Attestation – DIV – Client Back Office - Claudia Romero 08-18-2026.msg</t>
         </is>
       </c>
       <c r="C11" s="64" t="inlineStr">
@@ -13400,7 +13498,7 @@
       </c>
       <c r="D11" s="64" t="inlineStr">
         <is>
-          <t>RE_ Management Attestation – OFAC.msg</t>
+          <t>RE_ Management Attestation – DIV Client Back Office.msg</t>
         </is>
       </c>
       <c r="E11" s="64" t="inlineStr">
@@ -13415,22 +13513,22 @@
       </c>
       <c r="G11" s="64" t="inlineStr">
         <is>
-          <t>08/19/2026 – David Marquez</t>
+          <t>08/18/2026 – Claudia Romero</t>
         </is>
       </c>
       <c r="H11" s="64" t="inlineStr">
         <is>
-          <t>Cesar Vidal request to Department Managers (08/17/2026; DR exercises 11/15/2025 and 02/21/2026; BCiC export attached) and David Marquez (OFAC Manager) reply. Attachment: Data_Integrity_Attestation_Santander-BCiC (005) - BSA-AML-OFAC Compliance.pdf – signed OFAC Manager, VP, BSA/AML-OFAC Compliance, 8/19/2026. Attestation §1: IT DR team facilitates DIV annually; §2: 63 entries / 13 applications, all Y/Y/Y; §3.5: retained in BCMS/BCiC; §3.6: contemporaneous approval going forward.</t>
+          <t>Claudia Romero (Client Back Office Manager VP) returns the signed Management Attestation – attachment: Data_Integrity_Attestation_Santander-BCiC (002).pdf (signed Claudia Romero).</t>
         </is>
       </c>
       <c r="I11" s="64" t="inlineStr">
         <is>
-          <t>1822, 1867, 1868, 3299, 4052, 3301, 1903, 1917, 1936, 1937</t>
+          <t>1822, 1867, 1868, 3299, 1937</t>
         </is>
       </c>
       <c r="J11" s="64" t="inlineStr">
         <is>
-          <t>B, C, G, H, J, L, M, N, O, P</t>
+          <t>G, H, J, O</t>
         </is>
       </c>
       <c r="K11" s="64" t="inlineStr"/>
@@ -13439,12 +13537,12 @@
     <row r="12" ht="34.5" customHeight="1" s="71">
       <c r="A12" s="64" t="inlineStr">
         <is>
-          <t>DMA03</t>
+          <t>DMA02</t>
         </is>
       </c>
       <c r="B12" s="64" t="inlineStr">
         <is>
-          <t>DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg</t>
+          <t>DMA02_RE_ Management Attestation – DIV – BSA-AML-OFAC Compliance - David Marquez 08-19-2026.msg</t>
         </is>
       </c>
       <c r="C12" s="64" t="inlineStr">
@@ -13454,7 +13552,7 @@
       </c>
       <c r="D12" s="64" t="inlineStr">
         <is>
-          <t>Management Attestation – DIV Payment &amp; Cash Management.msg</t>
+          <t>RE_ Management Attestation – OFAC.msg</t>
         </is>
       </c>
       <c r="E12" s="64" t="inlineStr">
@@ -13469,22 +13567,22 @@
       </c>
       <c r="G12" s="64" t="inlineStr">
         <is>
-          <t>08/18/2026 – Frank Puentes</t>
+          <t>08/19/2026 – David Marquez</t>
         </is>
       </c>
       <c r="H12" s="64" t="inlineStr">
         <is>
-          <t>Frank Puentes returns the signed attestation – attachment: 4069_001.pdf (scan, signed Executive Director, Payments &amp; Cash Management, 8/18/2026).</t>
+          <t>Cesar Vidal request to Department Managers (08/17/2026; DR exercises 11/15/2025 and 02/21/2026; BCiC export attached) and David Marquez (OFAC Manager) reply. Attachment: Data_Integrity_Attestation_Santander-BCiC (005) - BSA-AML-OFAC Compliance.pdf – signed OFAC Manager, VP, BSA/AML-OFAC Compliance, 8/19/2026. Attestation §1: IT DR team facilitates DIV annually; §2: 63 entries / 13 applications, all Y/Y/Y; §3.5: retained in BCMS/BCiC; §3.6: contemporaneous approval going forward.</t>
         </is>
       </c>
       <c r="I12" s="64" t="inlineStr">
         <is>
-          <t>3301, 1903, 1937</t>
+          <t>1822, 1867, 1868, 3299, 4052, 3301, 1903, 1917, 1936, 1937</t>
         </is>
       </c>
       <c r="J12" s="64" t="inlineStr">
         <is>
-          <t>G, H, J, O</t>
+          <t>B, C, G, H, J, L, M, N, O, P</t>
         </is>
       </c>
       <c r="K12" s="64" t="inlineStr"/>
@@ -13493,12 +13591,12 @@
     <row r="13" ht="34.5" customHeight="1" s="71">
       <c r="A13" s="64" t="inlineStr">
         <is>
-          <t>DMA04</t>
+          <t>DMA03</t>
         </is>
       </c>
       <c r="B13" s="64" t="inlineStr">
         <is>
-          <t>DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg</t>
+          <t>DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg</t>
         </is>
       </c>
       <c r="C13" s="64" t="inlineStr">
@@ -13508,7 +13606,7 @@
       </c>
       <c r="D13" s="64" t="inlineStr">
         <is>
-          <t>RE_ Management Attestation – DIV Investment Operations.msg</t>
+          <t>Management Attestation – DIV Payment &amp; Cash Management.msg</t>
         </is>
       </c>
       <c r="E13" s="64" t="inlineStr">
@@ -13523,17 +13621,17 @@
       </c>
       <c r="G13" s="64" t="inlineStr">
         <is>
-          <t>08/17/2026 – Michelle Oropesa</t>
+          <t>08/18/2026 – Frank Puentes</t>
         </is>
       </c>
       <c r="H13" s="64" t="inlineStr">
         <is>
-          <t>Michelle Oropesa (Investment Operations Director) returns the signed attestation – attachment: Data_Integrity_Attestation_Santander-BCiC.pdf (signed Investment Operations Director, VP, 8/17/2026).</t>
+          <t>Frank Puentes returns the signed attestation – attachment: 4069_001.pdf (scan, signed Executive Director, Payments &amp; Cash Management, 8/18/2026).</t>
         </is>
       </c>
       <c r="I13" s="64" t="inlineStr">
         <is>
-          <t>4052, 1936, 1937</t>
+          <t>3301, 1903, 1937</t>
         </is>
       </c>
       <c r="J13" s="64" t="inlineStr">
@@ -13547,12 +13645,12 @@
     <row r="14" ht="34.5" customHeight="1" s="71">
       <c r="A14" s="64" t="inlineStr">
         <is>
-          <t>DMA05</t>
+          <t>DMA04</t>
         </is>
       </c>
       <c r="B14" s="64" t="inlineStr">
         <is>
-          <t>DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg</t>
+          <t>DMA04_RE_ Management Attestation – DIV – Investment Operations - Michelle Oropesa 08-17-2026.msg</t>
         </is>
       </c>
       <c r="C14" s="64" t="inlineStr">
@@ -13562,7 +13660,7 @@
       </c>
       <c r="D14" s="64" t="inlineStr">
         <is>
-          <t>RE_ Management Attestation – DIV Operations.msg</t>
+          <t>RE_ Management Attestation – DIV Investment Operations.msg</t>
         </is>
       </c>
       <c r="E14" s="64" t="inlineStr">
@@ -13577,17 +13675,17 @@
       </c>
       <c r="G14" s="64" t="inlineStr">
         <is>
-          <t>08/19/2026 – Maria Teresa (Mayte) Del Cerro</t>
+          <t>08/17/2026 – Michelle Oropesa</t>
         </is>
       </c>
       <c r="H14" s="64" t="inlineStr">
         <is>
-          <t>Senior Director of Operations returns the signed attestation – attachments: Data_Integrity_Attestation_Santander-BCiC.pdf (signed Maria Teresa Del Cerro Hontanilla, Director of Operations, 08/19/2026) and the BCiC export (same file as E16b).</t>
+          <t>Michelle Oropesa (Investment Operations Director) returns the signed attestation – attachment: Data_Integrity_Attestation_Santander-BCiC.pdf (signed Investment Operations Director, VP, 8/17/2026).</t>
         </is>
       </c>
       <c r="I14" s="64" t="inlineStr">
         <is>
-          <t>3299, 1903, 1937</t>
+          <t>4052, 1936, 1937</t>
         </is>
       </c>
       <c r="J14" s="64" t="inlineStr">
@@ -13601,12 +13699,12 @@
     <row r="15" ht="34.5" customHeight="1" s="71">
       <c r="A15" s="64" t="inlineStr">
         <is>
-          <t>DMA06</t>
+          <t>DMA05</t>
         </is>
       </c>
       <c r="B15" s="64" t="inlineStr">
         <is>
-          <t>DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg</t>
+          <t>DMA05_RE_ Management Attestation – DIV – Operations (Governance &amp; Static Data, Multi-Family Office) - Maria Teresa Del Cerro 08-19-2026.msg</t>
         </is>
       </c>
       <c r="C15" s="64" t="inlineStr">
@@ -13616,7 +13714,7 @@
       </c>
       <c r="D15" s="64" t="inlineStr">
         <is>
-          <t>RE_ Management Attestation – DIV Trading and Capital Markets.msg</t>
+          <t>RE_ Management Attestation – DIV Operations.msg</t>
         </is>
       </c>
       <c r="E15" s="64" t="inlineStr">
@@ -13631,17 +13729,17 @@
       </c>
       <c r="G15" s="64" t="inlineStr">
         <is>
-          <t>08/18/2026 – Ricardo Garcia-Marques</t>
+          <t>08/19/2026 – Maria Teresa (Mayte) Del Cerro</t>
         </is>
       </c>
       <c r="H15" s="64" t="inlineStr">
         <is>
-          <t>Attestation and approval from Trading &amp; Capital Markets (covers BCiC records approved by Ricardo Garcia) – attachment: Data_Integrity_Attestation_Santander-BCiC_signed.pdf (e-signed MD, Head of Trading &amp; Capital Markets, 08/18/2026 11:45 AM EDT).</t>
+          <t>Senior Director of Operations returns the signed attestation – attachments: Data_Integrity_Attestation_Santander-BCiC.pdf (signed Maria Teresa Del Cerro Hontanilla, Director of Operations, 08/19/2026) and the BCiC export (same file as E16b).</t>
         </is>
       </c>
       <c r="I15" s="64" t="inlineStr">
         <is>
-          <t>1937</t>
+          <t>3299, 1903, 1937</t>
         </is>
       </c>
       <c r="J15" s="64" t="inlineStr">
@@ -13655,12 +13753,12 @@
     <row r="16" ht="23" customHeight="1" s="71">
       <c r="A16" s="64" t="inlineStr">
         <is>
-          <t>DMA07</t>
+          <t>DMA06</t>
         </is>
       </c>
       <c r="B16" s="64" t="inlineStr">
         <is>
-          <t>DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg</t>
+          <t>DMA06_RE_ Management Attestation – DIV – Trading &amp; Capital Markets (AIS, Portfolio Advisory, P&amp;I Tech) - Ricardo Garcia-Marques 08-18-2026.msg</t>
         </is>
       </c>
       <c r="C16" s="64" t="inlineStr">
@@ -13670,7 +13768,7 @@
       </c>
       <c r="D16" s="64" t="inlineStr">
         <is>
-          <t>RE_ Management Attestation – DIV Treasury and Capital Planning.msg</t>
+          <t>RE_ Management Attestation – DIV Trading and Capital Markets.msg</t>
         </is>
       </c>
       <c r="E16" s="64" t="inlineStr">
@@ -13685,12 +13783,12 @@
       </c>
       <c r="G16" s="64" t="inlineStr">
         <is>
-          <t>08/18/2026 – Martha Sullivan</t>
+          <t>08/18/2026 – Ricardo Garcia-Marques</t>
         </is>
       </c>
       <c r="H16" s="64" t="inlineStr">
         <is>
-          <t>Martha Sullivan returns the signed attestation – attachment: Data_Integrity_Attestation_Santander-BCiC.pdf (signed Balance Sheet Manager, Treasury).</t>
+          <t>Attestation and approval from Trading &amp; Capital Markets (covers BCiC records approved by Ricardo Garcia) – attachment: Data_Integrity_Attestation_Santander-BCiC_signed.pdf (e-signed MD, Head of Trading &amp; Capital Markets, 08/18/2026 11:45 AM EDT).</t>
         </is>
       </c>
       <c r="I16" s="64" t="inlineStr">
@@ -13709,12 +13807,12 @@
     <row r="17" ht="23" customHeight="1" s="71">
       <c r="A17" s="64" t="inlineStr">
         <is>
-          <t>DMA08</t>
+          <t>DMA07</t>
         </is>
       </c>
       <c r="B17" s="64" t="inlineStr">
         <is>
-          <t>DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg</t>
+          <t>DMA07_RE_ Management Attestation – DIV – Treasury &amp; Capital Planning - Martha Sullivan 08-18-2026.msg</t>
         </is>
       </c>
       <c r="C17" s="64" t="inlineStr">
@@ -13724,7 +13822,7 @@
       </c>
       <c r="D17" s="64" t="inlineStr">
         <is>
-          <t>RE_ Management Attestation – DIV Solvency and Market Risk.msg</t>
+          <t>RE_ Management Attestation – DIV Treasury and Capital Planning.msg</t>
         </is>
       </c>
       <c r="E17" s="64" t="inlineStr">
@@ -13734,17 +13832,17 @@
       </c>
       <c r="F17" s="64" t="inlineStr">
         <is>
-          <t>Email approval</t>
+          <t>Email attestation</t>
         </is>
       </c>
       <c r="G17" s="64" t="inlineStr">
         <is>
-          <t>08/18/2026 – Ivan Caisapanta</t>
+          <t>08/18/2026 – Martha Sullivan</t>
         </is>
       </c>
       <c r="H17" s="64" t="inlineStr">
         <is>
-          <t>"Hi Elizabeth, You have my approval" – Financial Risk (BCiC Department Manager recorded as Xavier Caisapanta).</t>
+          <t>Martha Sullivan returns the signed attestation – attachment: Data_Integrity_Attestation_Santander-BCiC.pdf (signed Balance Sheet Manager, Treasury).</t>
         </is>
       </c>
       <c r="I17" s="64" t="inlineStr">
@@ -13763,12 +13861,12 @@
     <row r="18" ht="23" customHeight="1" s="71">
       <c r="A18" s="64" t="inlineStr">
         <is>
-          <t>DMA09</t>
+          <t>DMA08</t>
         </is>
       </c>
       <c r="B18" s="64" t="inlineStr">
         <is>
-          <t>DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg</t>
+          <t>DMA08_RE_ Management Attestation – DIV – Solvency &amp; Market Risk (Financial Risk) - Ivan Caisapanta 08-18-2026.msg</t>
         </is>
       </c>
       <c r="C18" s="64" t="inlineStr">
@@ -13778,7 +13876,7 @@
       </c>
       <c r="D18" s="64" t="inlineStr">
         <is>
-          <t>RE_ Management Attestation – DIV General Services.msg</t>
+          <t>RE_ Management Attestation – DIV Solvency and Market Risk.msg</t>
         </is>
       </c>
       <c r="E18" s="64" t="inlineStr">
@@ -13788,17 +13886,17 @@
       </c>
       <c r="F18" s="64" t="inlineStr">
         <is>
-          <t>Email attestation</t>
+          <t>Email approval</t>
         </is>
       </c>
       <c r="G18" s="64" t="inlineStr">
         <is>
-          <t>08/18/2026 – Clara G. De Castro</t>
+          <t>08/18/2026 – Ivan Caisapanta</t>
         </is>
       </c>
       <c r="H18" s="64" t="inlineStr">
         <is>
-          <t>Clara De Castro (Director, General Services &amp; Facilities) returns the signed attestation – attachment: Data_Integrity_Attestation_Santander-BCiC.pdf (signed Clara G. De Castro).</t>
+          <t>"Hi Elizabeth, You have my approval" – Financial Risk (BCiC Department Manager recorded as Xavier Caisapanta).</t>
         </is>
       </c>
       <c r="I18" s="64" t="inlineStr">
@@ -13817,12 +13915,12 @@
     <row r="19" ht="23" customHeight="1" s="71">
       <c r="A19" s="64" t="inlineStr">
         <is>
-          <t>DMA10</t>
+          <t>DMA09</t>
         </is>
       </c>
       <c r="B19" s="64" t="inlineStr">
         <is>
-          <t>DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml</t>
+          <t>DMA09_RE_ Management Attestation – DIV – General Services (Marketing &amp; General Services) - Clara De Castro 08-18-2026.msg</t>
         </is>
       </c>
       <c r="C19" s="64" t="inlineStr">
@@ -13832,7 +13930,7 @@
       </c>
       <c r="D19" s="64" t="inlineStr">
         <is>
-          <t>RE Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises).eml</t>
+          <t>RE_ Management Attestation – DIV General Services.msg</t>
         </is>
       </c>
       <c r="E19" s="64" t="inlineStr">
@@ -13842,17 +13940,17 @@
       </c>
       <c r="F19" s="64" t="inlineStr">
         <is>
-          <t>Email approval</t>
+          <t>Email attestation</t>
         </is>
       </c>
       <c r="G19" s="64" t="inlineStr">
         <is>
-          <t>08/21/2026 – Victoria Fernandez</t>
+          <t>08/18/2026 – Clara G. De Castro</t>
         </is>
       </c>
       <c r="H19" s="64" t="inlineStr">
         <is>
-          <t>"Approved" – Digital Wealth.</t>
+          <t>Clara De Castro (Director, General Services &amp; Facilities) returns the signed attestation – attachment: Data_Integrity_Attestation_Santander-BCiC.pdf (signed Clara G. De Castro).</t>
         </is>
       </c>
       <c r="I19" s="64" t="inlineStr">
@@ -13871,12 +13969,12 @@
     <row r="20" ht="23" customHeight="1" s="71">
       <c r="A20" s="64" t="inlineStr">
         <is>
-          <t>DMA11</t>
+          <t>DMA10</t>
         </is>
       </c>
       <c r="B20" s="64" t="inlineStr">
         <is>
-          <t>DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml</t>
+          <t>DMA10_RE_ Management Attestation – DIV – Digital Wealth - Victoria Fernandez 08-21-2026.eml</t>
         </is>
       </c>
       <c r="C20" s="64" t="inlineStr">
@@ -13886,7 +13984,7 @@
       </c>
       <c r="D20" s="64" t="inlineStr">
         <is>
-          <t>RE Management Attestation – DIV Commercial Middle Office.eml</t>
+          <t>RE Management Attestation – Data Integrity Validation Testing (November 2025 &amp; February 2026 Exercises).eml</t>
         </is>
       </c>
       <c r="E20" s="64" t="inlineStr">
@@ -13901,17 +13999,17 @@
       </c>
       <c r="G20" s="64" t="inlineStr">
         <is>
-          <t>09/09/2026 – Miguel Orozco</t>
+          <t>08/21/2026 – Victoria Fernandez</t>
         </is>
       </c>
       <c r="H20" s="64" t="inlineStr">
         <is>
-          <t>"I approve the integrity validation for the testing performed by the Commercial Middle Office."</t>
+          <t>"Approved" – Digital Wealth.</t>
         </is>
       </c>
       <c r="I20" s="64" t="inlineStr">
         <is>
-          <t>3299, 1937</t>
+          <t>1937</t>
         </is>
       </c>
       <c r="J20" s="64" t="inlineStr">
@@ -13925,12 +14023,12 @@
     <row r="21" ht="23" customHeight="1" s="71">
       <c r="A21" s="64" t="inlineStr">
         <is>
-          <t>DMA12</t>
+          <t>DMA11</t>
         </is>
       </c>
       <c r="B21" s="64" t="inlineStr">
         <is>
-          <t>DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml</t>
+          <t>DMA11_RE_ Management Attestation – DIV – Commercial Middle Office - Miguel Orozco 09-09-2026.eml</t>
         </is>
       </c>
       <c r="C21" s="64" t="inlineStr">
@@ -13940,7 +14038,7 @@
       </c>
       <c r="D21" s="64" t="inlineStr">
         <is>
-          <t>RE Management Attestation – DIV Client Servicing Unit.eml</t>
+          <t>RE Management Attestation – DIV Commercial Middle Office.eml</t>
         </is>
       </c>
       <c r="E21" s="64" t="inlineStr">
@@ -13955,17 +14053,17 @@
       </c>
       <c r="G21" s="64" t="inlineStr">
         <is>
-          <t>09/09/2026 – Liliana Vizhnay</t>
+          <t>09/09/2026 – Miguel Orozco</t>
         </is>
       </c>
       <c r="H21" s="64" t="inlineStr">
         <is>
-          <t>"I approve." – Client Servicing Unit.</t>
+          <t>"I approve the integrity validation for the testing performed by the Commercial Middle Office."</t>
         </is>
       </c>
       <c r="I21" s="64" t="inlineStr">
         <is>
-          <t>1937</t>
+          <t>3299, 1937</t>
         </is>
       </c>
       <c r="J21" s="64" t="inlineStr">
@@ -13979,12 +14077,12 @@
     <row r="22" ht="23" customHeight="1" s="71">
       <c r="A22" s="64" t="inlineStr">
         <is>
-          <t>DMA13</t>
+          <t>DMA12</t>
         </is>
       </c>
       <c r="B22" s="64" t="inlineStr">
         <is>
-          <t>DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml</t>
+          <t>DMA12_RE_ Management Attestation – DIV – Client Servicing Unit - Liliana Vizhnay 09-09-2026.eml</t>
         </is>
       </c>
       <c r="C22" s="64" t="inlineStr">
@@ -13994,7 +14092,7 @@
       </c>
       <c r="D22" s="64" t="inlineStr">
         <is>
-          <t>RE Management Attestation – DIV Unified Communication - Cisco Call Manager.eml</t>
+          <t>RE Management Attestation – DIV Client Servicing Unit.eml</t>
         </is>
       </c>
       <c r="E22" s="64" t="inlineStr">
@@ -14009,22 +14107,22 @@
       </c>
       <c r="G22" s="64" t="inlineStr">
         <is>
-          <t>09/09/2026 – Elizabeth Noda</t>
+          <t>09/09/2026 – Liliana Vizhnay</t>
         </is>
       </c>
       <c r="H22" s="64" t="inlineStr">
         <is>
-          <t>"approve" – Cisco Call Manager (IT). Cisco Call Manager is NOT one of the 10 tested applications – retained for completeness only.</t>
+          <t>"I approve." – Client Servicing Unit.</t>
         </is>
       </c>
       <c r="I22" s="64" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1937</t>
         </is>
       </c>
       <c r="J22" s="64" t="inlineStr">
         <is>
-          <t>Supplemental</t>
+          <t>G, H, J, O</t>
         </is>
       </c>
       <c r="K22" s="64" t="inlineStr"/>
@@ -14033,52 +14131,52 @@
     <row r="23" ht="23" customHeight="1" s="71">
       <c r="A23" s="64" t="inlineStr">
         <is>
-          <t>E01</t>
+          <t>DMA13</t>
         </is>
       </c>
       <c r="B23" s="64" t="inlineStr">
         <is>
-          <t>BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx</t>
+          <t>DMA13_RE_ Management Attestation – DIV – IT Unified Communication - Cisco Call Manager - Elizabeth Noda 09-09-2026 (out of scope).eml</t>
         </is>
       </c>
       <c r="C23" s="64" t="inlineStr">
         <is>
-          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
+          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals</t>
         </is>
       </c>
       <c r="D23" s="64" t="inlineStr">
         <is>
-          <t>Applications In Scope for DR Test BSI (13).xlsx</t>
+          <t>RE Management Attestation – DIV Unified Communication - Cisco Call Manager.eml</t>
         </is>
       </c>
       <c r="E23" s="64" t="inlineStr">
         <is>
-          <t>Data Integrity &amp; Email Testing Evidence.zip</t>
+          <t>DIV Manager Attestation Email_Approvals.zip</t>
         </is>
       </c>
       <c r="F23" s="64" t="inlineStr">
         <is>
-          <t>BCiC export</t>
+          <t>Email approval</t>
         </is>
       </c>
       <c r="G23" s="64" t="inlineStr">
         <is>
-          <t>BCiC – Applications In Scope for DR Test BSI</t>
+          <t>09/09/2026 – Elizabeth Noda</t>
         </is>
       </c>
       <c r="H23" s="64" t="inlineStr">
         <is>
-          <t>BCiC export of the BSI DR-scope population (43 applications) with Exercise Date and 2025 DR / Backup-Restore / DIV scope flags.</t>
+          <t>"approve" – Cisco Call Manager (IT). Cisco Call Manager is NOT one of the 10 tested applications – retained for completeness only.</t>
         </is>
       </c>
       <c r="I23" s="64" t="inlineStr">
         <is>
-          <t>1822, 1867, 1868, 3299, 4052, 3301, 1903, 1917, 1936, 1937</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J23" s="64" t="inlineStr">
         <is>
-          <t>B, C, D, K, L, N</t>
+          <t>Supplemental</t>
         </is>
       </c>
       <c r="K23" s="64" t="inlineStr"/>
@@ -14087,12 +14185,12 @@
     <row r="24" ht="23" customHeight="1" s="71">
       <c r="A24" s="64" t="inlineStr">
         <is>
-          <t>E02</t>
+          <t>E01</t>
         </is>
       </c>
       <c r="B24" s="64" t="inlineStr">
         <is>
-          <t>BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg</t>
+          <t>BSI.IT.6.C7.3_E01_Applications In Scope for DR Test BSI (13).xlsx</t>
         </is>
       </c>
       <c r="C24" s="64" t="inlineStr">
@@ -14102,7 +14200,7 @@
       </c>
       <c r="D24" s="64" t="inlineStr">
         <is>
-          <t>screenshot BCiC apps in scope for DR Testing.jpg</t>
+          <t>Applications In Scope for DR Test BSI (13).xlsx</t>
         </is>
       </c>
       <c r="E24" s="64" t="inlineStr">
@@ -14112,17 +14210,17 @@
       </c>
       <c r="F24" s="64" t="inlineStr">
         <is>
-          <t>BCiC screenshot</t>
+          <t>BCiC export</t>
         </is>
       </c>
       <c r="G24" s="64" t="inlineStr">
         <is>
-          <t>09/10/2026 – Cesar Vidal</t>
+          <t>BCiC – Applications In Scope for DR Test BSI</t>
         </is>
       </c>
       <c r="H24" s="64" t="inlineStr">
         <is>
-          <t>BCiC Applications screen with view 'Applications In Scope for DR Test BSI' selected (1–20 of 43 items).</t>
+          <t>BCiC export of the BSI DR-scope population (43 applications) with Exercise Date and 2025 DR / Backup-Restore / DIV scope flags.</t>
         </is>
       </c>
       <c r="I24" s="64" t="inlineStr">
@@ -14132,7 +14230,7 @@
       </c>
       <c r="J24" s="64" t="inlineStr">
         <is>
-          <t>D, K, N</t>
+          <t>B, C, D, K, L, N</t>
         </is>
       </c>
       <c r="K24" s="64" t="inlineStr"/>
@@ -14141,12 +14239,12 @@
     <row r="25" ht="23" customHeight="1" s="71">
       <c r="A25" s="64" t="inlineStr">
         <is>
-          <t>E03</t>
+          <t>E02</t>
         </is>
       </c>
       <c r="B25" s="64" t="inlineStr">
         <is>
-          <t>BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
+          <t>BSI.IT.6.C7.3_E02_screenshot BCiC apps in scope for DR Testing.jpg</t>
         </is>
       </c>
       <c r="C25" s="64" t="inlineStr">
@@ -14156,7 +14254,7 @@
       </c>
       <c r="D25" s="64" t="inlineStr">
         <is>
-          <t>All Data Integrity Validation Testing_FV.xls</t>
+          <t>screenshot BCiC apps in scope for DR Testing.jpg</t>
         </is>
       </c>
       <c r="E25" s="64" t="inlineStr">
@@ -14166,17 +14264,17 @@
       </c>
       <c r="F25" s="64" t="inlineStr">
         <is>
-          <t>BCiC export</t>
+          <t>BCiC screenshot</t>
         </is>
       </c>
       <c r="G25" s="64" t="inlineStr">
         <is>
-          <t>BCiC – Data Integrity Validation Testing (62 records)</t>
+          <t>09/10/2026 – Cesar Vidal</t>
         </is>
       </c>
       <c r="H25" s="64" t="inlineStr">
         <is>
-          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Y/N Format/Headers/Content, Attestation Date / Provided By. Row numbers quoted are Excel rows.</t>
+          <t>BCiC Applications screen with view 'Applications In Scope for DR Test BSI' selected (1–20 of 43 items).</t>
         </is>
       </c>
       <c r="I25" s="64" t="inlineStr">
@@ -14186,7 +14284,7 @@
       </c>
       <c r="J25" s="64" t="inlineStr">
         <is>
-          <t>B, C, D, E, F, G, H, I, K, L, M, O, P</t>
+          <t>D, K, N</t>
         </is>
       </c>
       <c r="K25" s="64" t="inlineStr"/>
@@ -14195,12 +14293,12 @@
     <row r="26">
       <c r="A26" s="64" t="inlineStr">
         <is>
-          <t>E04</t>
+          <t>E03</t>
         </is>
       </c>
       <c r="B26" s="64" t="inlineStr">
         <is>
-          <t>BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg</t>
+          <t>BSI.IT.6.C7.3_E03_All Data Integrity Validation Testing_FV.xls</t>
         </is>
       </c>
       <c r="C26" s="64" t="inlineStr">
@@ -14210,7 +14308,7 @@
       </c>
       <c r="D26" s="64" t="inlineStr">
         <is>
-          <t>BCiC_Screenshot for Data Integrity Validation report.jpg</t>
+          <t>All Data Integrity Validation Testing_FV.xls</t>
         </is>
       </c>
       <c r="E26" s="64" t="inlineStr">
@@ -14220,17 +14318,17 @@
       </c>
       <c r="F26" s="64" t="inlineStr">
         <is>
-          <t>BCiC screenshot</t>
+          <t>BCiC export</t>
         </is>
       </c>
       <c r="G26" s="64" t="inlineStr">
         <is>
-          <t>09/10/2026 – Cesar Vidal</t>
+          <t>BCiC – Data Integrity Validation Testing (62 records)</t>
         </is>
       </c>
       <c r="H26" s="64" t="inlineStr">
         <is>
-          <t>BCiC 'Data Integrity Validation Testing' screen (1–20 of 66 items) showing tester, validation date, manager, approval date, Y/N results and attestation fields.</t>
+          <t>BCiC DIV export incl. Business Tester, Business Data Validation Date, Department Manager, Department Manager Approval Date, Y/N Format/Headers/Content, Attestation Date / Provided By. Row numbers quoted are Excel rows.</t>
         </is>
       </c>
       <c r="I26" s="64" t="inlineStr">
@@ -14240,7 +14338,7 @@
       </c>
       <c r="J26" s="64" t="inlineStr">
         <is>
-          <t>D, E, F, G, H, K, P</t>
+          <t>B, C, D, E, F, G, H, I, K, L, M, O, P</t>
         </is>
       </c>
       <c r="K26" s="64" t="inlineStr"/>
@@ -14249,12 +14347,12 @@
     <row r="27">
       <c r="A27" s="64" t="inlineStr">
         <is>
-          <t>E05</t>
+          <t>E04</t>
         </is>
       </c>
       <c r="B27" s="64" t="inlineStr">
         <is>
-          <t>BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg</t>
+          <t>BSI.IT.6.C7.3_E04_BCiC_Screenshot for Data Integrity Validation report.jpg</t>
         </is>
       </c>
       <c r="C27" s="64" t="inlineStr">
@@ -14264,7 +14362,7 @@
       </c>
       <c r="D27" s="64" t="inlineStr">
         <is>
-          <t>IT BIA Results Review and preparation for DR .msg</t>
+          <t>BCiC_Screenshot for Data Integrity Validation report.jpg</t>
         </is>
       </c>
       <c r="E27" s="64" t="inlineStr">
@@ -14274,17 +14372,17 @@
       </c>
       <c r="F27" s="64" t="inlineStr">
         <is>
-          <t>Meeting invite</t>
+          <t>BCiC screenshot</t>
         </is>
       </c>
       <c r="G27" s="64" t="inlineStr">
         <is>
-          <t>09/15/2025 – Elizabeth Noda</t>
+          <t>09/10/2026 – Cesar Vidal</t>
         </is>
       </c>
       <c r="H27" s="64" t="inlineStr">
         <is>
-          <t>IT DR meeting invite to review the 2025 BIA results and applications list ahead of the DR exercise (same invite re-sent 09/18/2025 – duplicate E06 removed).</t>
+          <t>BCiC 'Data Integrity Validation Testing' screen (1–20 of 66 items) showing tester, validation date, manager, approval date, Y/N results and attestation fields.</t>
         </is>
       </c>
       <c r="I27" s="64" t="inlineStr">
@@ -14294,7 +14392,7 @@
       </c>
       <c r="J27" s="64" t="inlineStr">
         <is>
-          <t>M, N</t>
+          <t>D, E, F, G, H, K, P</t>
         </is>
       </c>
       <c r="K27" s="64" t="inlineStr"/>
@@ -14303,12 +14401,12 @@
     <row r="28">
       <c r="A28" s="64" t="inlineStr">
         <is>
-          <t>E07</t>
+          <t>E05</t>
         </is>
       </c>
       <c r="B28" s="64" t="inlineStr">
         <is>
-          <t>BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg</t>
+          <t>BSI.IT.6.C7.3_E05_IT BIA Results Review and preparation for DR .msg</t>
         </is>
       </c>
       <c r="C28" s="64" t="inlineStr">
@@ -14318,7 +14416,7 @@
       </c>
       <c r="D28" s="64" t="inlineStr">
         <is>
-          <t>DATA INTERITY FILS FROM 111425.msg</t>
+          <t>IT BIA Results Review and preparation for DR .msg</t>
         </is>
       </c>
       <c r="E28" s="64" t="inlineStr">
@@ -14328,27 +14426,27 @@
       </c>
       <c r="F28" s="64" t="inlineStr">
         <is>
-          <t>Email + report attachments</t>
+          <t>Meeting invite</t>
         </is>
       </c>
       <c r="G28" s="64" t="inlineStr">
         <is>
-          <t>11/15/2025 – Frank Puentes</t>
+          <t>09/15/2025 – Elizabeth Noda</t>
         </is>
       </c>
       <c r="H28" s="64" t="inlineStr">
         <is>
-          <t>Pre-DR (11/14/2025) source reports: Fedlink, OFAC ACH/FED/SWIFT, Payment Monitor, SWIFT Interface Monitor, outgoing Fedwire/SWIFT. Embedded attachments: FEDLINK INCOMING FEDWIRES 111425 0523PM.pdf; FEDLINK OUTGOING FEDWIRES 111425 0523PM.pdf; OFAC ACH 111425 0512PM.pdf; OFAC FED 111425 0511PM.pdf; OFAC SWIFT 111425 0511PM.pdf; OUTGOING FEDWIRE 111425 506PM.xls; OUTGOING SWIFT 111425 509PM.xls; PAYMENT MONITOR INCOMING FEDWIRE 111425 516PM PG1.pdf; PAYMENT MONITOR INCOMING FEDWIRE 111425 516PM PG2.pdf; PAYMENT MONITOR OUTGOING FEDWIRE 111425 516PM PG1.pdf; PAYMENT MONITOR OUTGOING FEDWIRE 111425 516PM PG2.pdf; SWIFT INTERFACE MONITOR 111425 519PM.pdf; SWIFT INTERFACE MONITOR 111425 520PM 2ND SAMPLE.pdf.</t>
+          <t>IT DR meeting invite to review the 2025 BIA results and applications list ahead of the DR exercise (same invite re-sent 09/18/2025 – duplicate E06 removed).</t>
         </is>
       </c>
       <c r="I28" s="64" t="inlineStr">
         <is>
-          <t>3301, 1903, 1936, 1937</t>
+          <t>1822, 1867, 1868, 3299, 4052, 3301, 1903, 1917, 1936, 1937</t>
         </is>
       </c>
       <c r="J28" s="64" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M, N</t>
         </is>
       </c>
       <c r="K28" s="64" t="inlineStr"/>
@@ -14357,12 +14455,12 @@
     <row r="29">
       <c r="A29" s="64" t="inlineStr">
         <is>
-          <t>E08</t>
+          <t>E07</t>
         </is>
       </c>
       <c r="B29" s="64" t="inlineStr">
         <is>
-          <t>BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg</t>
+          <t>BSI.IT.6.C7.3_E07_DATA INTERITY FILS FROM 111425.msg</t>
         </is>
       </c>
       <c r="C29" s="64" t="inlineStr">
@@ -14372,7 +14470,7 @@
       </c>
       <c r="D29" s="64" t="inlineStr">
         <is>
-          <t>FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg</t>
+          <t>DATA INTERITY FILS FROM 111425.msg</t>
         </is>
       </c>
       <c r="E29" s="64" t="inlineStr">
@@ -14392,7 +14490,7 @@
       </c>
       <c r="H29" s="64" t="inlineStr">
         <is>
-          <t>DR test-day (11/15/2025) re-run of the same reports for comparison with 11/14/2025 source. Embedded attachments: FEDLINK INCOMING FEDWIRES 111425 -1115 1148AM.pdf; FEDLINK OUTGOINT TRANSFERS 114125 - 111525 1144AM.pdf; OFAC ACH 111425 - 11152025 1126AM.pdf; OFAC FED 111425 - 111525 1126AM.pdf; OFAC SWIFT 111425 - 111525 1128AM.pdf; OUTGOING FEDWIRE 111525 1025AM.xls; OUTGOING SWIFT 111525 1026AM.xls; PAYMENT MONITOR 111424 - 111525 PG 11156AM.pdf; PAYMENT MONITOR 111425 - 111525 PG 2 1158AM.pdf; PAYMENT MONITOR OUTGOING 111425 - 111525 PG 1 1156AM.pdf; PAYMENT MONITOR OUTGOING 111425 - 111525 PG 2 1156AM.pdf; SWIFT INTERFACE MONITOR INCOMING MT103 111425 - 111525 1152AM.pdf; SWIFT INTERFACE MONITOR INCOMING MT199 111425 -111525 1152AM.pdf.</t>
+          <t>Pre-DR (11/14/2025) source reports: Fedlink, OFAC ACH/FED/SWIFT, Payment Monitor, SWIFT Interface Monitor, outgoing Fedwire/SWIFT. Embedded attachments: FEDLINK INCOMING FEDWIRES 111425 0523PM.pdf; FEDLINK OUTGOING FEDWIRES 111425 0523PM.pdf; OFAC ACH 111425 0512PM.pdf; OFAC FED 111425 0511PM.pdf; OFAC SWIFT 111425 0511PM.pdf; OUTGOING FEDWIRE 111425 506PM.xls; OUTGOING SWIFT 111425 509PM.xls; PAYMENT MONITOR INCOMING FEDWIRE 111425 516PM PG1.pdf; PAYMENT MONITOR INCOMING FEDWIRE 111425 516PM PG2.pdf; PAYMENT MONITOR OUTGOING FEDWIRE 111425 516PM PG1.pdf; PAYMENT MONITOR OUTGOING FEDWIRE 111425 516PM PG2.pdf; SWIFT INTERFACE MONITOR 111425 519PM.pdf; SWIFT INTERFACE MONITOR 111425 520PM 2ND SAMPLE.pdf.</t>
         </is>
       </c>
       <c r="I29" s="64" t="inlineStr">
@@ -14402,7 +14500,7 @@
       </c>
       <c r="J29" s="64" t="inlineStr">
         <is>
-          <t>F, M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="K29" s="64" t="inlineStr"/>
@@ -14411,12 +14509,12 @@
     <row r="30">
       <c r="A30" s="64" t="inlineStr">
         <is>
-          <t>E09</t>
+          <t>E08</t>
         </is>
       </c>
       <c r="B30" s="64" t="inlineStr">
         <is>
-          <t>BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg</t>
+          <t>BSI.IT.6.C7.3_E08_FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg</t>
         </is>
       </c>
       <c r="C30" s="64" t="inlineStr">
@@ -14426,7 +14524,7 @@
       </c>
       <c r="D30" s="64" t="inlineStr">
         <is>
-          <t>RE_ Yearly Backup and restore exercise (Client Back Office)</t>
+          <t>FILES FROM 111525 DR TEST - DATA COMPARISON FROM 111425.msg</t>
         </is>
       </c>
       <c r="E30" s="64" t="inlineStr">
@@ -14436,27 +14534,27 @@
       </c>
       <c r="F30" s="64" t="inlineStr">
         <is>
-          <t>Email approval</t>
+          <t>Email + report attachments</t>
         </is>
       </c>
       <c r="G30" s="64" t="inlineStr">
         <is>
-          <t>03/03/2026 – 05/05/2026 – Claudia Romero</t>
+          <t>11/15/2025 – Frank Puentes</t>
         </is>
       </c>
       <c r="H30" s="64" t="inlineStr">
         <is>
-          <t>Client Back Office test evidence (Mariorly Morales, Ilumel Rodriguez, Rolando Bonilla) and Claudia Romero "Approved." 05/05/2026. Thread maps ACH Express, FedExport, FedImport, Imaging101 to Client Back Office / Claudia Romero.</t>
+          <t>DR test-day (11/15/2025) re-run of the same reports for comparison with 11/14/2025 source. Embedded attachments: FEDLINK INCOMING FEDWIRES 111425 -1115 1148AM.pdf; FEDLINK OUTGOINT TRANSFERS 114125 - 111525 1144AM.pdf; OFAC ACH 111425 - 11152025 1126AM.pdf; OFAC FED 111425 - 111525 1126AM.pdf; OFAC SWIFT 111425 - 111525 1128AM.pdf; OUTGOING FEDWIRE 111525 1025AM.xls; OUTGOING SWIFT 111525 1026AM.xls; PAYMENT MONITOR 111424 - 111525 PG 11156AM.pdf; PAYMENT MONITOR 111425 - 111525 PG 2 1158AM.pdf; PAYMENT MONITOR OUTGOING 111425 - 111525 PG 1 1156AM.pdf; PAYMENT MONITOR OUTGOING 111425 - 111525 PG 2 1156AM.pdf; SWIFT INTERFACE MONITOR INCOMING MT103 111425 - 111525 1152AM.pdf; SWIFT INTERFACE MONITOR INCOMING MT199 111425 -111525 1152AM.pdf.</t>
         </is>
       </c>
       <c r="I30" s="64" t="inlineStr">
         <is>
-          <t>1822, 1867, 1868, 3299, 1937</t>
+          <t>3301, 1903, 1936, 1937</t>
         </is>
       </c>
       <c r="J30" s="64" t="inlineStr">
         <is>
-          <t>E, G, H, J, M, N, O</t>
+          <t>F, M</t>
         </is>
       </c>
       <c r="K30" s="64" t="inlineStr"/>
@@ -14465,12 +14563,12 @@
     <row r="31">
       <c r="A31" s="64" t="inlineStr">
         <is>
-          <t>E10</t>
+          <t>E09</t>
         </is>
       </c>
       <c r="B31" s="64" t="inlineStr">
         <is>
-          <t>BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg</t>
+          <t>BSI.IT.6.C7.3_E09_RE_ Yearly Backup and restore exercise- client back office sign off-ACH,ACH Express, FedExport, FedImport,Imagi.msg</t>
         </is>
       </c>
       <c r="C31" s="64" t="inlineStr">
@@ -14480,7 +14578,7 @@
       </c>
       <c r="D31" s="64" t="inlineStr">
         <is>
-          <t>RE_ Yearly Backup and restore exercise-- re-run (Finance)</t>
+          <t>RE_ Yearly Backup and restore exercise (Client Back Office)</t>
         </is>
       </c>
       <c r="E31" s="64" t="inlineStr">
@@ -14495,22 +14593,22 @@
       </c>
       <c r="G31" s="64" t="inlineStr">
         <is>
-          <t>03/09/2026 – Lina Acuna</t>
+          <t>03/03/2026 – 05/05/2026 – Claudia Romero</t>
         </is>
       </c>
       <c r="H31" s="64" t="inlineStr">
         <is>
-          <t>Finance DIV results chart (Jose Acero) and Lina Acuna "Approved" 03/09/2026 (T24 / ReconXpert backup-restore).</t>
+          <t>Client Back Office test evidence (Mariorly Morales, Ilumel Rodriguez, Rolando Bonilla) and Claudia Romero "Approved." 05/05/2026. Thread maps ACH Express, FedExport, FedImport, Imaging101 to Client Back Office / Claudia Romero.</t>
         </is>
       </c>
       <c r="I31" s="64" t="inlineStr">
         <is>
-          <t>1917, 1937</t>
+          <t>1822, 1867, 1868, 3299, 1937</t>
         </is>
       </c>
       <c r="J31" s="64" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>E, G, H, J, M, N, O</t>
         </is>
       </c>
       <c r="K31" s="64" t="inlineStr"/>
@@ -14519,12 +14617,12 @@
     <row r="32">
       <c r="A32" s="64" t="inlineStr">
         <is>
-          <t>E13</t>
+          <t>E10</t>
         </is>
       </c>
       <c r="B32" s="64" t="inlineStr">
         <is>
-          <t>BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg</t>
+          <t>BSI.IT.6.C7.3_E10_RE_ Yearly Backup and restore exercise-- re-run- Finance approval-T24-ReconXpert.msg</t>
         </is>
       </c>
       <c r="C32" s="64" t="inlineStr">
@@ -14534,7 +14632,7 @@
       </c>
       <c r="D32" s="64" t="inlineStr">
         <is>
-          <t>miasx2 T24 environment(s) miaeod miabed01 refreshed correctly.msg</t>
+          <t>RE_ Yearly Backup and restore exercise-- re-run (Finance)</t>
         </is>
       </c>
       <c r="E32" s="64" t="inlineStr">
@@ -14544,27 +14642,27 @@
       </c>
       <c r="F32" s="64" t="inlineStr">
         <is>
-          <t>System email</t>
+          <t>Email approval</t>
         </is>
       </c>
       <c r="G32" s="64" t="inlineStr">
         <is>
-          <t>11/13/2024 – T24 backup user</t>
+          <t>03/09/2026 – Lina Acuna</t>
         </is>
       </c>
       <c r="H32" s="64" t="inlineStr">
         <is>
-          <t>T24 environment refresh log – prior period (outside review period); supplemental only.</t>
+          <t>Finance DIV results chart (Jose Acero) and Lina Acuna "Approved" 03/09/2026 (T24 / ReconXpert backup-restore).</t>
         </is>
       </c>
       <c r="I32" s="64" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1917, 1937</t>
         </is>
       </c>
       <c r="J32" s="64" t="inlineStr">
         <is>
-          <t>Supplemental</t>
+          <t>M</t>
         </is>
       </c>
       <c r="K32" s="64" t="inlineStr"/>
@@ -14573,12 +14671,12 @@
     <row r="33">
       <c r="A33" s="64" t="inlineStr">
         <is>
-          <t>E16b</t>
+          <t>E13</t>
         </is>
       </c>
       <c r="B33" s="64" t="inlineStr">
         <is>
-          <t>BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+          <t>BSI.IT.6.C7.3_E13_miasx2 T24 environment(s)  miaeod miabed01 refreshed correctly.msg</t>
         </is>
       </c>
       <c r="C33" s="64" t="inlineStr">
@@ -14588,7 +14686,7 @@
       </c>
       <c r="D33" s="64" t="inlineStr">
         <is>
-          <t>All Data Integrity Validation Testing-BSI 2025-26.xlsx (attachment of DMA05 email)</t>
+          <t>miasx2 T24 environment(s) miaeod miabed01 refreshed correctly.msg</t>
         </is>
       </c>
       <c r="E33" s="64" t="inlineStr">
@@ -14598,52 +14696,88 @@
       </c>
       <c r="F33" s="64" t="inlineStr">
         <is>
-          <t>BCiC export</t>
+          <t>System email</t>
         </is>
       </c>
       <c r="G33" s="64" t="inlineStr">
         <is>
-          <t>08/2026 – BCiC export sent with attestation request</t>
+          <t>11/13/2024 – T24 backup user</t>
         </is>
       </c>
       <c r="H33" s="64" t="inlineStr">
         <is>
-          <t>BCiC DIV export 2025-26 (64 rows; no manager columns) sent to managers with the attestation request and returned by M. T. Del Cerro (DMA05). Row numbers are Excel rows.</t>
+          <t>T24 environment refresh log – prior period (outside review period); supplemental only.</t>
         </is>
       </c>
       <c r="I33" s="64" t="inlineStr">
         <is>
-          <t>1822, 1867, 1868, 3299, 4052, 3301, 1903, 1917, 1936, 1937</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J33" s="64" t="inlineStr">
         <is>
-          <t>B, D, E, F, I, K, P</t>
+          <t>Supplemental</t>
         </is>
       </c>
       <c r="K33" s="64" t="inlineStr"/>
       <c r="L33" s="82" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="82" t="n"/>
-      <c r="B34" s="82" t="n"/>
-      <c r="C34" s="82" t="n"/>
-      <c r="D34" s="82" t="n"/>
-      <c r="E34" s="82" t="n"/>
-      <c r="F34" s="82" t="n"/>
-      <c r="G34" s="82" t="n"/>
-      <c r="H34" s="82" t="n"/>
-      <c r="I34" s="82" t="n"/>
-      <c r="J34" s="82" t="n"/>
-      <c r="K34" s="82" t="n"/>
+      <c r="A34" s="64" t="inlineStr">
+        <is>
+          <t>E16b</t>
+        </is>
+      </c>
+      <c r="B34" s="64" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3_E16b_All Data Integrity Validation Testing-BSI 2025-26.xlsx</t>
+        </is>
+      </c>
+      <c r="C34" s="64" t="inlineStr">
+        <is>
+          <t>BSI.IT.6.C7.3-Evidences\04_Data_Integrity_and_Email_Testing_Evidence</t>
+        </is>
+      </c>
+      <c r="D34" s="64" t="inlineStr">
+        <is>
+          <t>All Data Integrity Validation Testing-BSI 2025-26.xlsx (attachment of DMA05 email)</t>
+        </is>
+      </c>
+      <c r="E34" s="64" t="inlineStr">
+        <is>
+          <t>Data Integrity &amp; Email Testing Evidence.zip</t>
+        </is>
+      </c>
+      <c r="F34" s="64" t="inlineStr">
+        <is>
+          <t>BCiC export</t>
+        </is>
+      </c>
+      <c r="G34" s="64" t="inlineStr">
+        <is>
+          <t>08/2026 – BCiC export sent with attestation request</t>
+        </is>
+      </c>
+      <c r="H34" s="64" t="inlineStr">
+        <is>
+          <t>BCiC DIV export 2025-26 (64 rows; no manager columns) sent to managers with the attestation request and returned by M. T. Del Cerro (DMA05). Row numbers are Excel rows.</t>
+        </is>
+      </c>
+      <c r="I34" s="64" t="inlineStr">
+        <is>
+          <t>1822, 1867, 1868, 3299, 4052, 3301, 1903, 1917, 1936, 1937</t>
+        </is>
+      </c>
+      <c r="J34" s="64" t="inlineStr">
+        <is>
+          <t>B, D, E, F, I, K, P</t>
+        </is>
+      </c>
+      <c r="K34" s="64" t="inlineStr"/>
       <c r="L34" s="82" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="60" t="inlineStr">
-        <is>
-          <t>Redundant files removed from the repository (one copy of each item retained)</t>
-        </is>
-      </c>
+      <c r="A35" s="82" t="n"/>
       <c r="B35" s="82" t="n"/>
       <c r="C35" s="82" t="n"/>
       <c r="D35" s="82" t="n"/>
@@ -14657,31 +14791,15 @@
       <c r="L35" s="82" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Removed item</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Former location</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Retained ref</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Retained file location</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Reason</t>
-        </is>
-      </c>
+      <c r="A36" s="60" t="inlineStr">
+        <is>
+          <t>Redundant files removed from the repository (one copy of each item retained)</t>
+        </is>
+      </c>
+      <c r="B36" s="82" t="n"/>
+      <c r="C36" s="82" t="n"/>
+      <c r="D36" s="82" t="n"/>
+      <c r="E36" s="82" t="n"/>
       <c r="F36" s="82" t="n"/>
       <c r="G36" s="82" t="n"/>
       <c r="H36" s="82" t="n"/>
@@ -14691,29 +14809,29 @@
       <c r="L36" s="82" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="64" t="inlineStr">
-        <is>
-          <t>MA02</t>
-        </is>
-      </c>
-      <c r="B37" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\01_Management_Attestation_In-Scope_Applications\MA02_RE_ Management Attestation – DIV Testing (Nov 2025 &amp; Feb 2026) – Payments &amp; Cash Management – Frank Puentes 08-18-2026.msg</t>
-        </is>
-      </c>
-      <c r="C37" s="64" t="inlineStr">
-        <is>
-          <t>DMA03</t>
-        </is>
-      </c>
-      <c r="D37" s="64" t="inlineStr">
-        <is>
-          <t>BSI.IT.6.C7.3-Evidences\03_DIV_Manager_Attestation_Email_Approvals\DMA03_RE_ Management Attestation – DIV – Payments &amp; Cash Management - Frank Puentes 08-18-2026.msg</t>
-        </is>
-      </c>
-      <c r="E37" s="64" t="inlineStr">
-        <is>
-          <t>same email message (subject, sent 08/18/2026 14:50, attachment 4069_001.pdf)</t>
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Removed item</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Former location</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Retained ref</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Retained file location</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Reason</t>
         </is>
       </c>
       <c r="F37" s="82" t="n"/>
@@ -16327,7 +16445,7 @@
       <c r="L120" s="82" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:K33"/>
+  <autoFilter ref="A2:K34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>